<commit_message>
Refresh E5.2 validation workbook
</commit_message>
<xml_diff>
--- a/docs/E5.2_Resultados_Validacion_Componentes.xlsx
+++ b/docs/E5.2_Resultados_Validacion_Componentes.xlsx
@@ -3476,7 +3476,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed e integrado al dashboard 2026-05-06</t>
+          <t>Automatizado / passed e integrado al dashboard 2026-05-06</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / DS-UI-AMH-01 con evidencias verificables marked passed 2026-05-06</t>
+          <t>Automatizado / DS-UI-AMH-01 con evidencias verificables marked passed 2026-05-06</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / DS-UI-SV-01 y SV-GTFS-BENCH-04 passed</t>
+          <t>Automatizado / DS-UI-SV-01 y SV-GTFS-BENCH-04 passed</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed</t>
+          <t>Automatizado / passed</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed</t>
+          <t>Automatizado / passed</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-07</t>
+          <t>Automatizado / passed 2026-05-07</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / API+UI passed</t>
+          <t>Automatizado / API+UI passed</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
@@ -4466,8 +4466,8 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Paso 1: Validar repo oficial gtfs-bench.
-Paso 2: Generar mini-fixture trazable.
+          <t>Paso 1: Validar repositorio oficial GTFS-Bench.
+Paso 2: Derivar muestra runtime trazable.
 Paso 3: Materializar RDF.
 Paso 4: Publicar RDF como HttpData.
 Paso 5: Registrar hashes/metadatos.</t>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Usar mini-fixture para validacion visual; dataset completo queda como ejecucion pesada opt-in.</t>
+          <t>Usar muestra runtime derivada para validación visual; el dataset completo puede quedar como ejecución pesada fuera de la validación habitual.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed</t>
+          <t>Automatizado / passed</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
@@ -4834,12 +4834,11 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Paso 1: Preparar dataset linguistico FLARES o mini-fixture trazable.
+          <t>Paso 1: Preparar dataset lingüístico FLARES trazable.
 Paso 2: Registrar modelo/endpoint como asset gobernado en INESData.
 Paso 3: Consumer descubre y negocia acceso.
-Paso 4: Abrir AI Model Browser/Execution/Benchmarking.
-Paso 5: Ejecutar o simular inferencia/benchmark.
-Paso 6: Registrar metricas y evidencia visual/API.</t>
+Paso 4: Abrir AI Model Browser/Execution/Benchmarking según corresponda.
+Paso 5: Registrar evidencia funcional e integración.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -5101,11 +5100,11 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/03-provider-setup.spec.ts
-validation/ui/core/03b-provider-policy-create.spec.ts
-validation/ui/core/03c-provider-contract-definition-create.spec.ts
-validation/ui/core/05-consumer-negotiation.spec.ts
-validation/ui/core/06-consumer-transfer.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/03-provider-setup.spec.ts
+validation/ui/adapters/inesdata/specs/03b-provider-policy-create.spec.ts
+validation/ui/adapters/inesdata/specs/03c-provider-contract-definition-create.spec.ts
+validation/ui/adapters/inesdata/specs/05-consumer-negotiation.spec.ts
+validation/ui/adapters/inesdata/specs/06-consumer-transfer.spec.ts</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -5185,8 +5184,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>Automatizado / opt-in
-Ejecucion INESData marcada passed 2026-05-06</t>
+          <t>Automatizado / ejecución INESData marcada passed 2026-05-06</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -5237,18 +5235,18 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>- Modelos FLARES-mini preparados
+          <t>- Modelos FLARES preparados
 - Dataset benchmark disponible
-- validacion visual UI activada</t>
+- Validación visual UI activada</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Paso 1: Abrir Model Benchmarking.
 Paso 2: Seleccionar FLARES Reliability Baseline A y B.
-Paso 3: Cargar FLARES-mini Local Benchmark Dataset.
+Paso 3: Cargar FLARES benchmark dataset.
 Paso 4: Click en Run Benchmark.
-Paso 5: Ver tabla de resultados, metricas y Best Model.</t>
+Paso 5: Ver tabla de resultados, métricas y Best Model.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -5263,7 +5261,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>Automatizado opt-in pasado 4/4</t>
+          <t>Automatizado / passed 4/4</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -5333,13 +5331,12 @@
       <c r="I8" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/dataspace_integration.py
-validation/ui/core/07-semantic-virtualization-httpdata.spec.ts</t>
+validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-06
-Ejecucion INESData marcada passed 2026-05-06</t>
+          <t>Automatizado / passed 2026-05-06 / Ejecución INESData marcada passed 2026-05-06</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -5392,7 +5389,7 @@
       <c r="F9" s="3" t="inlineStr">
         <is>
           <t>- Evidencia VS HttpData disponible
-- Fixture GTFS-Madrid-Bench-mini disponible</t>
+- Repositorio oficial GTFS-Madrid-Bench sincronizado</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -5489,13 +5486,13 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/08-ontology-hub-inesdata-readonly.spec.ts
-Activacion: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
+          <t>validation/ui/adapters/inesdata/specs/08-ontology-hub-inesdata-readonly.spec.ts
+Variable runtime: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-06</t>
+          <t>Automatizado / passed 2026-05-06</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -5569,14 +5566,13 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/09-ai-model-hub-httpdata.spec.ts
-Activacion: UI_AI_MODEL_HUB_HTTPDATA_DEMO=1</t>
+          <t>validation/ui/adapters/inesdata/specs/09-ai-model-hub-httpdata.spec.ts
+Variable runtime: UI_AI_MODEL_HUB_HTTPDATA_DEMO=1</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-06
-Ejecucion INESData marcada passed 2026-05-06</t>
+          <t>Automatizado / passed 2026-05-06 / Ejecución INESData marcada passed 2026-05-06</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -5771,7 +5767,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/01-login-readiness.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/01-login-readiness.spec.ts</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -5839,7 +5835,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/03-provider-setup.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/03-provider-setup.spec.ts</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -5906,7 +5902,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/03b-provider-policy-create.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/03b-provider-policy-create.spec.ts</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -5974,7 +5970,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/03c-provider-contract-definition-create.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/03c-provider-contract-definition-create.spec.ts</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -6042,7 +6038,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/04-consumer-catalog.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/04-consumer-catalog.spec.ts</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -6109,7 +6105,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/05-consumer-negotiation.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/05-consumer-negotiation.spec.ts</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -6177,7 +6173,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/06-consumer-transfer.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/06-consumer-transfer.spec.ts</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -6246,14 +6242,13 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/07-semantic-virtualization-httpdata.spec.ts
-Activacion: UI_SEMANTIC_VIRTUALIZATION_HTTPDATA_DEMO=1</t>
+          <t>validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts
+Variable runtime: UI_SEMANTIC_VIRTUALIZATION_HTTPDATA_DEMO=1</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-06
-Ejecucion INESData marcada passed 2026-05-06</t>
+          <t>Automatizado / passed 2026-05-06 / Ejecución INESData marcada passed 2026-05-06</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -6374,7 +6369,7 @@
           <t>- Consumer connector portal is reachable
 - Ontology Hub is deployed
 - Runtime config exposes ontologyUrl
-- UI_ONTOLOGY_HUB_INESDATA_DEMO=1 is enabled for this opt-in validacion visual</t>
+- UI_ONTOLOGY_HUB_INESDATA_DEMO=1 is enabled by the validation runner when required</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -6394,8 +6389,8 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/08-ontology-hub-inesdata-readonly.spec.ts
-Activacion: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
+          <t>validation/ui/adapters/inesdata/specs/08-ontology-hub-inesdata-readonly.spec.ts
+Variable runtime: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
@@ -7805,8 +7800,8 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/08-ontology-hub-inesdata-readonly.spec.ts
-Activacion: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
+          <t>validation/ui/adapters/inesdata/specs/08-ontology-hub-inesdata-readonly.spec.ts
+Variable runtime: UI_ONTOLOGY_HUB_INESDATA_DEMO=1</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -10981,7 +10976,7 @@
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/connector_governance_api.py
-Activacion: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -11131,7 +11126,7 @@
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/connector_governance_api.py
-Activacion: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -11192,9 +11187,9 @@
       <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Paso 1: Abrir AI Model Hub en la ruta de Model Benchmarking.
-Paso 2: Asegurar dos modelos FLARES-mini comparables en el contexto consumer.
+Paso 2: Asegurar dos modelos FLARES comparables en el contexto consumer.
 Paso 3: Seleccionar los modelos FLARES Reliability Baseline A y Baseline B.
-Paso 4: Verificar que el boton Run Benchmark queda habilitado.</t>
+Paso 4: Confirmar que ambos quedan listos para benchmarking.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -11206,7 +11201,7 @@
         <is>
           <t>validation/components/ai_model_hub/ui/specs/pt5_mh_12_15_model_benchmarking_demo.spec.js
 validation/components/ai_model_hub/model_benchmarking_api.py
-Activacion: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -11230,8 +11225,7 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>The runner selects two controlled FLARES-mini compatible model assets and records the benchmark-ready dataset mapping. The Playwright UI validacion visual reuses the same fixture and controlled infer route without touching AIModelHub sources.
-Ejecucion con evidencias verificables 2026-05-06: 4/4 Playwright passed para PT5-MH-12..15 con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye capturas, videos, reporte Playwright y dashboard local.</t>
+          <t>The runner selects two controlled FLARES-compatible model assets and records the benchmark-ready dataset mapping. The Playwright UI validation reuses the same fixture and controlled infer route without touching AIModelHub sources.</t>
         </is>
       </c>
     </row>
@@ -11269,10 +11263,10 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Cargar el dataset FLARES-mini Local Benchmark Dataset.
+          <t>Paso 1: Cargar el dataset FLARES benchmark.
 Paso 2: Mantener inputPath=input, expectedPath=expected_label y predictionPath=result.label.
 Paso 3: Click en Run Benchmark.
-Paso 4: Verificar que ambos modelos reciben las mismas filas de entrada.</t>
+Paso 4: Verificar que ambos modelos se ejecutan sobre los mismos inputs.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -11284,7 +11278,7 @@
         <is>
           <t>validation/components/ai_model_hub/ui/specs/pt5_mh_12_15_model_benchmarking_demo.spec.js
 validation/components/ai_model_hub/model_benchmarking_api.py
-Activacion: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -11308,8 +11302,7 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>The runner executes both controlled models over the same FLARES-mini input fingerprints and stores per-model execution evidence. The Playwright validacion visual clicks Run Benchmark and shows those executions in the UI.
-Ejecucion con evidencias verificables 2026-05-06: 4/4 Playwright passed para PT5-MH-12..15 con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye capturas, videos, reporte Playwright y dashboard local.</t>
+          <t>The runner executes both controlled models over the same FLARES input fingerprints and stores per-model execution evidence. The Playwright UI validation clicks Run Benchmark and shows those executions in the UI.</t>
         </is>
       </c>
     </row>
@@ -11361,7 +11354,7 @@
         <is>
           <t>validation/components/ai_model_hub/ui/specs/pt5_mh_12_15_model_benchmarking_demo.spec.js
 validation/components/ai_model_hub/model_benchmarking_api.py
-Activacion: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -11423,10 +11416,10 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Abrir la seccion Benchmark Results.
+          <t>Paso 1: Abrir la sección Benchmark Results.
 Paso 2: Verificar la tarjeta Best Model.
-Paso 3: Verificar que la tabla contiene los dos modelos FLARES-mini.
-Paso 4: Conservar screenshot, video y JSON de la validacion visual.</t>
+Paso 3: Verificar que la tabla contiene los dos modelos FLARES.
+Paso 4: Conservar screenshot, video y JSON de la validación visual.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -11438,7 +11431,7 @@
         <is>
           <t>validation/components/ai_model_hub/ui/specs/pt5_mh_12_15_model_benchmarking_demo.spec.js
 validation/components/ai_model_hub/model_benchmarking_api.py
-Activacion: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_MODEL_BENCHMARKING=1</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -11512,7 +11505,7 @@
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/connector_governance_api.py
-Activacion: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -11583,7 +11576,7 @@
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/connector_governance_api.py
-Activacion: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -11654,7 +11647,7 @@
       <c r="I24" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/connector_governance_api.py
-Activacion: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_CONNECTOR_GOVERNANCE=1</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -11691,7 +11684,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Linguistic domain use case with FLARES-mini</t>
+          <t>Linguistic domain use case with FLARES</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -11712,29 +11705,27 @@
       <c r="F25" s="3" t="inlineStr">
         <is>
           <t>- AI Model Hub, provider connector and consumer connector are deployed
-- FLARES-mini fixture is available in the framework</t>
+- FLARES source repository was synchronized by Level 5</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Publish FLARES-mini on demand as a provider dataset asset.
+          <t>Paso 1: Publish FLARES on demand as a provider dataset asset.
 Paso 2: Discover the published dataset from the consumer catalog.
 Paso 3: Negotiate the corresponding contract agreement from the consumer side.
-Paso 4: Bootstrap benchmark-ready linguistic models in the consumer.
-Paso 5: Load the FLARES benchmark dataset inside Model Benchmarking.
-Paso 6: Execute a FLARES-mini record through the connector-side model execution API.
-Paso 7: Link the execution evidence to expected_outputs.json for the future reliability-label assertion.</t>
+Paso 4: Prepare the linguistic benchmarking flow.
+Paso 5: Execute a FLARES payload through the connector-side model execution API.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>FLARES-mini can populate the dataspace on demand, reach a negotiated agreement, prepare the linguistic benchmarking flow and execute a FLARES payload through the connector API without requiring global seeding</t>
+          <t>FLARES can populate the dataspace on demand, reach a negotiated agreement, prepare the linguistic benchmarking flow and execute a FLARES payload through the connector API without requiring global seeding.</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/functional/specs/mh_ling_01_flares_reliability.spec.js
-validation/components/ai_model_hub/model_execution_api.py --flares-mini</t>
+validation/components/ai_model_hub/model_execution_api.py --flares-dataset</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -11756,7 +11747,7 @@
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>Opt-in scaffold for Phase 3. The current automated slice covers provider publication, consumer negotiation and benchmark-ready dataset/model linkage; connector-side model execution is validated through the PT5-MH-10 runner with --flares-mini. The semantic FLARES reliability-label comparison remains pending until a FLARES-compatible model endpoint is available.</t>
+          <t>Phase 3 scaffold executed from Level 6. The current automated slice covers provider publication, consumer negotiation and benchmark-ready dataset/model linkage; connector-side model execution is validated through PT5-MH-10 with --flares-dataset.</t>
         </is>
       </c>
     </row>
@@ -11768,7 +11759,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Mobility domain use case with GTFS-Madrid-Bench-mini</t>
+          <t>Mobility domain use case with GTFS-Madrid-Bench</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11788,23 +11779,21 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>- GTFS-Madrid-Bench-mini fixture is available in the framework
+          <t>- GTFS-Madrid-Bench source repository was synchronized by Level 5
 - At least two controlled mobility benchmark models are selected by the suite</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Cargar metadata, schema, sample y expected_outputs de GTFS-Madrid-Bench-mini.
+          <t>Paso 1: Cargar metadata, schema, sample y expected_outputs derivados de GTFS-Madrid-Bench.
 Paso 2: Validar join keys GTFS-like para stops, routes, trips y stop_times.
-Paso 3: Construir filas deterministas desde transfer_benchmark_cases.
-Paso 4: Ejecutar modelos controlados de estimacion de ruta/ETA.
-Paso 5: Comparar secuencia de ruta y duracion esperada contra expected_outputs.json.
-Paso 6: Generar ranking, tabla y datos de graficas para una futura validacion visual de Model Benchmarking.</t>
+Paso 3: Construir filas deterministas desde el repositorio oficial sincronizado.
+Paso 4: Ejecutar benchmarking de movilidad y registrar métricas.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>GTFS-Madrid-Bench-mini produce evidencia reproducible de benchmarking de movilidad con joins validados, rutas/duraciones esperadas y metricas ranqueadas por modelo.</t>
+          <t>GTFS-Madrid-Bench produce evidencia reproducible de benchmarking de movilidad con joins validados, rutas/duraciones esperadas y métricas ranqueadas por modelo.</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -11818,7 +11807,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / passed 2026-05-06</t>
+          <t>Automatizado / passed 2026-05-06</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -11836,7 +11825,7 @@
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>Suite conservadora: no toca el repo AIModelHub local ni muta INESData. Cierra el contrato funcional de movilidad con fixture determinista hasta que exista ruta UI/API viva estable.</t>
+          <t>Suite conservadora: no toca el repo AIModelHub local ni muta INESData. Cierra el contrato funcional de movilidad con una muestra runtime derivada del repositorio oficial hasta que exista ruta UI/API viva estable.</t>
         </is>
       </c>
     </row>
@@ -11889,7 +11878,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/09-ai-model-hub-httpdata.spec.ts</t>
+          <t>validation/ui/adapters/inesdata/specs/09-ai-model-hub-httpdata.spec.ts</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -11913,8 +11902,7 @@
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>Linked cases: PT5-MH-03, PT5-MH-08, PT5-MH-09, PT5-MH-10, PT5-MH-18. validacion visual opt-in porque crea negociacion/acuerdo; evidencia final r8 ya esta integrada al dashboard local del framework.
-Ejecucion con evidencias verificables 2026-05-06: DS-UI-AMH-01 1/1 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; provider publica modelo HttpData, consumer lo descubre, abre detalle/ofertas y negocia desde INESData UI.</t>
+          <t>Linked cases: PT5-MH-03, PT5-MH-08, PT5-MH-09, PT5-MH-10, PT5-MH-18. Validación visual con creación controlada de negociación/acuerdo; evidencia final r8 ya está integrada al dashboard local del framework.</t>
         </is>
       </c>
     </row>
@@ -11966,14 +11954,14 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/10-ai-model-observer.spec.ts
-Activacion: UI_AI_MODEL_OBSERVER_DEMO=1
+          <t>validation/ui/adapters/inesdata/specs/10-ai-model-observer.spec.ts
+Variable runtime: UI_AI_MODEL_OBSERVER_DEMO=1
 Marcadores: PLAYWRIGHT_INTERACTION_MARKERS=1</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / ejecutado 2026-05-07 / skipped controlado por UI Observer no integrada</t>
+          <t>Automatizado / ejecutado 2026-05-07 / skipped controlado por UI Observer no integrada</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -12046,13 +12034,13 @@
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/model_observer_api.py
-Activacion: AI_MODEL_HUB_ENABLE_MODEL_OBSERVER=1
-Configuracion opcional: AI_MODEL_HUB_OBSERVER_API_BASE_URL=&lt;backend-url&gt;</t>
+Variable runtime: AI_MODEL_HUB_ENABLE_MODEL_OBSERVER=1
+Configuración opcional: AI_MODEL_HUB_OBSERVER_API_BASE_URL=&lt;backend-url&gt;</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Automatizado opt-in / ejecutado 2026-05-07 / skipped controlado por Observer API no disponible</t>
+          <t>Automatizado / ejecutado 2026-05-07 / skipped controlado por Observer API no disponible</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -12692,7 +12680,7 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: mappings RML/R2RML</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -12709,8 +12697,7 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; Level 6 ejecuta validation/components/semantic_virtualization/mapping_validation.py por defecto.</t>
         </is>
       </c>
     </row>
@@ -12843,7 +12830,7 @@
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: consulta multisource</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -12860,8 +12847,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la evidencia se genera mediante mapping_validation.py.</t>
         </is>
       </c>
     </row>
@@ -12917,7 +12903,7 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: consulta compleja</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -12934,8 +12920,7 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la suite valida forma, filtros y resultado esperado.</t>
         </is>
       </c>
     </row>
@@ -12991,7 +12976,7 @@
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: validación de mappings</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -13008,8 +12993,7 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la suite comprueba mapping válido e inválido controlado.</t>
         </is>
       </c>
     </row>
@@ -13041,13 +13025,13 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>- Ontología mobility-mini cargada como fixture
+          <t>- Ontología de movilidad controlada disponible como fixture
 - Fuentes de datos y términos semánticos disponibles</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Cargar fuente de datos y ontología mobility-mini.
+          <t>Paso 1: Cargar fuente de datos y ontología de movilidad controlada.
 Paso 2: Ejecutar el mapping que referencia términos de la ontología.
 Paso 3: Verificar que la salida usa los términos semánticos esperados.</t>
         </is>
@@ -13064,7 +13048,7 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: mappings con fuentes y ontologías</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -13081,8 +13065,7 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; se mantiene como fixture de validación del componente, no como dataset reducido de dominio.</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13097,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
+          <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible en el puerto configurado</t>
         </is>
       </c>
@@ -13133,8 +13116,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+          <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -13157,13 +13139,7 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Actualizacion 2026-05-06: el spec usa helpers live-marker para resaltar clicks, entradas, tabs y checkpoints visuales con PLAYWRIGHT_INTERACTION_MARKERS=1.
-Ejecucion con evidencias verificables 2026-05-06: 8/8 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye screenshots, videos, trazas, reporte Playwright y dashboard local.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in
-Marcadores visuales Playwright estandarizados 2026-05-06
-Ejecucion UI marcada passed 2026-05-06
-Computado en 00_Resumen como parte de la primera suite UI revisada del virtualizador: 8/8 passed.</t>
+          <t>Reconciliado 2026-05-18: la UI del mapping-editor se ejecuta en Level 6 dentro de la suite del componente; Kafka es el único bloque que requiere activación explícita por coste temporal. Evidencia previa: 8/8 Playwright passed con marcadores visuales.</t>
         </is>
       </c>
     </row>
@@ -13195,7 +13171,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
+          <t>- mapping-editor habilitado por la validación del componente
 - Mapping de ejemplo cargado en la UI</t>
         </is>
       </c>
@@ -13214,13 +13190,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+          <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Automatizado / revisado: entrada de ejecucion visible</t>
+          <t>Automatizado / revisado: entrada de ejecución visible</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -13238,13 +13213,7 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Actualizacion 2026-05-06: el spec usa helpers live-marker para resaltar clicks, entradas, tabs y checkpoints visuales con PLAYWRIGHT_INTERACTION_MARKERS=1.
-Ejecucion con evidencias verificables 2026-05-06: 8/8 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye screenshots, videos, trazas, reporte Playwright y dashboard local.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in
-Marcadores visuales Playwright estandarizados 2026-05-06
-Ejecucion UI marcada passed 2026-05-06
-Computado en 00_Resumen como parte de la primera suite UI revisada del virtualizador: 8/8 passed.</t>
+          <t>Reconciliado 2026-05-18: la entrada de ejecución/materialización del editor está automatizada en la suite UI del componente y se ejecuta por defecto cuando el componente está configurado.</t>
         </is>
       </c>
     </row>
@@ -13300,7 +13269,7 @@
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: exportación RML/R2RML</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -13317,8 +13286,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la suite parsea el artefacto exportable como RML/R2RML Turtle.</t>
         </is>
       </c>
     </row>
@@ -13374,7 +13342,7 @@
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: evaluación de métodos</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -13391,8 +13359,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la suite compara métodos con criterios reproducibles.</t>
         </is>
       </c>
     </row>
@@ -13444,13 +13411,13 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/07-semantic-virtualization-httpdata.spec.ts
+          <t>validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts
 validation/components/semantic_virtualization/dataspace_integration.py</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Automatizado / revisado: integracion INESData HttpData</t>
+          <t>Automatizado / revisado: integración INESData HttpData</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -13469,12 +13436,7 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>DS-UI-SV-01 confirma desde UI de INESData que el motor virtualizado se publica como HttpData, se descubre y se negocia.
-Ejecucion con evidencias verificables 2026-05-06: DS-UI-SV-01 1/1 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; provider publica asset HttpData del virtualizador, consumer lo descubre, abre detalle/ofertas y negocia desde INESData UI.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-06
-Ejecucion INESData marcada passed 2026-05-06
-Computado en 00_Resumen como el caso de integracion revisado del virtualizador con INESData.</t>
+          <t>Reconciliado 2026-05-18: DS-UI-SV-01 confirma desde UI de INESData que el motor virtualizado se publica como HttpData, se descubre y se negocia. La ruta Playwright actual es validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts.</t>
         </is>
       </c>
     </row>
@@ -13530,7 +13492,7 @@
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: errores controlados</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -13547,8 +13509,7 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado</t>
+          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; runner.py valida respuesta HTTP 4xx controlada ante consulta inválida.</t>
         </is>
       </c>
     </row>
@@ -13580,7 +13541,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
+          <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible</t>
         </is>
       </c>
@@ -13600,7 +13561,7 @@
       <c r="I19" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -13622,14 +13583,7 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>Refuerza PT5-VS-06/PT5-VS-07 como validacion visual sin importar ontologias reales ni mutar recursos persistentes.
-Actualizacion 2026-05-06: el spec usa helpers live-marker para resaltar clicks, entradas, tabs y checkpoints visuales con PLAYWRIGHT_INTERACTION_MARKERS=1.
-Ejecucion con evidencias verificables 2026-05-06: 8/8 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye screenshots, videos, trazas, reporte Playwright y dashboard local.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-06
-Marcadores visuales Playwright estandarizados 2026-05-06
-Ejecucion UI marcada passed 2026-05-06
-Computado en 00_Resumen como parte de la primera suite UI revisada del virtualizador: 8/8 passed.</t>
+          <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-06/PT5-VS-07; evidencia previa con marcadores visuales Playwright.</t>
         </is>
       </c>
     </row>
@@ -13661,8 +13615,8 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
-- Sesion Streamlit nueva para la prueba</t>
+          <t>- mapping-editor habilitado por la validación del componente
+- Sesión Streamlit nueva para la prueba</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -13683,7 +13637,7 @@
       <c r="I20" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -13705,14 +13659,7 @@
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Refuerza PT5-VS-01, PT5-VS-05 y PT5-VS-06; la mutacion queda limitada a la sesion del navegador de Streamlit.
-Actualizacion 2026-05-06: el spec usa helpers live-marker para resaltar clicks, entradas, tabs y checkpoints visuales con PLAYWRIGHT_INTERACTION_MARKERS=1.
-Ejecucion con evidencias verificables 2026-05-06: 8/8 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye screenshots, videos, trazas, reporte Playwright y dashboard local.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-06
-Marcadores visuales Playwright estandarizados 2026-05-06
-Ejecucion UI marcada passed 2026-05-06
-Computado en 00_Resumen como parte de la primera suite UI revisada del virtualizador: 8/8 passed.</t>
+          <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-01, PT5-VS-05 y PT5-VS-06; la mutación queda limitada a la sesión del navegador.</t>
         </is>
       </c>
     </row>
@@ -13744,8 +13691,8 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
-- Mapping temporal creado en sesion</t>
+          <t>- mapping-editor habilitado por la validación del componente
+- Mapping temporal creado en sesión</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -13766,7 +13713,7 @@
       <c r="I21" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -13788,14 +13735,7 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>Refuerza PT5-VS-08 y PT5-VS-09 como validacion visual; no ejecuta Morph-KGC si no hay fuentes de datos configuradas.
-Actualizacion 2026-05-06: el spec usa helpers live-marker para resaltar clicks, entradas, tabs y checkpoints visuales con PLAYWRIGHT_INTERACTION_MARKERS=1.
-Ejecucion con evidencias verificables 2026-05-06: 8/8 Playwright passed con PLAYWRIGHT_INTERACTION_MARKERS=1; incluye screenshots, videos, trazas, reporte Playwright y dashboard local.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-06
-Marcadores visuales Playwright estandarizados 2026-05-06
-Ejecucion UI marcada passed 2026-05-06
-Computado en 00_Resumen como parte de la primera suite UI revisada del virtualizador: 8/8 passed.</t>
+          <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-08 y PT5-VS-09; no requiere ejecutar Morph-KGC si no hay fuentes configuradas.</t>
         </is>
       </c>
     </row>
@@ -13827,9 +13767,9 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
+          <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible
-- Sesion Streamlit nueva para la prueba</t>
+- Sesión Streamlit nueva para la prueba</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -13853,12 +13793,12 @@
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: namespace y exportación desde editor</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -13875,9 +13815,7 @@
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>Level 5 quedo succeeded y el mapping-editor se valido via port-forward temporal. El spec usa Enter tras rellenar campos Streamlit para mostrar Bind/Export.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Passed opt-in / evidencia visual generada 2026-05-07</t>
+          <t>Reconciliado 2026-05-18: SV-UI-07 está catalogado como automated/mapped y la evidencia visual se generó en 2026-05-07; Level 6 lo incorpora dentro de la suite UI del componente.</t>
         </is>
       </c>
     </row>
@@ -13909,19 +13847,19 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>- mapping-editor habilitado como opt-in
+          <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible
-- Fixtures mobility-mini.owl y stops.csv disponibles en el framework</t>
+- Fixtures de ontología y CSV disponibles en el framework</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al URL del mapping-editor.
 Paso 2: Abrir Global Configuration.
-Paso 3: Crear un mapping temporal para aislar la sesion.
+Paso 3: Crear un mapping temporal para aislar la sesión.
 Paso 4: Abrir Ontologies.
-Paso 5: Seleccionar la opcion File e importar mobility-mini.owl.
-Paso 6: Click en Add y verificar que la ontologia queda disponible.
+Paso 5: Importar la ontología de movilidad controlada.
+Paso 6: Click en Add y verificar que la ontología queda disponible.
 Paso 7: Abrir Explore Ontology y capturar clases/propiedades visibles.
 Paso 8: Abrir Data Files.
 Paso 9: Subir stops.csv y click en Save.
@@ -13936,12 +13874,12 @@
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: importación de ontología y CSV</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -13958,9 +13896,7 @@
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>Level 5 ya despliega el mapping-editor. La evidencia se genero via port-forward temporal. Se usa mobility-mini.owl porque el uploader Streamlit rechazaba el MIME text/turtle de la fixture TTL antes de parsearla.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Passed opt-in / evidencia visual generada 2026-05-07</t>
+          <t>Reconciliado 2026-05-18: SV-UI-08 está catalogado como automated/mapped; usa fixtures controlados del componente para validar la UI sin versionar datasets reducidos de dominio.</t>
         </is>
       </c>
     </row>
@@ -13993,8 +13929,8 @@
       <c r="F24" s="3" t="inlineStr">
         <is>
           <t>- mapping-editor desplegado y accesible
-- Fixture RML no vacia compatible con el editor
-- Ontologia mobility-mini.owl disponible</t>
+- Fixture RML no vacía compatible con el editor
+- Ontología de movilidad controlada disponible</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -14004,11 +13940,11 @@
 Paso 3: Seleccionar "File" en "Import Existing Mapping".
 Paso 4: Subir "mapping_editor_mobility_network.rml.ttl".
 Paso 5: Escribir un label temporal para el mapping y click en "Import".
-Paso 6: Click en "Ontologies" y seleccionar importacion desde "File".
-Paso 7: Subir "mobility-mini.owl" y click en "Add".
+Paso 6: Click en "Ontologies" y seleccionar importación desde "File".
+Paso 7: Subir la ontología de movilidad controlada y click en "Add".
 Paso 8: Click en "Explore Mapping" y validar "Network Visualisation".
 Paso 9: Click en "Predefined Searches" y consultar "TriplesMaps", "Subject Maps" y "Predicate-Object Maps".
-Paso 10: Click en "Preview" y verificar la serializacion del mapping.
+Paso 10: Click en "Preview" y verificar la serialización del mapping.
 Paso 11: Click en "Ontology-Mapping Lens".
 Paso 12: Revisar "Mapping Composition", "Class Usage", "Property Usage" y "External Terms".</t>
         </is>
@@ -14021,13 +13957,13 @@
       <c r="I24" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
-Activacion: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1
+Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1
 Marcadores: PLAYWRIGHT_INTERACTION_MARKERS=1</t>
         </is>
       </c>
       <c r="J24" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: mapping no vacío y Ontology-Mapping Lens</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -14045,10 +13981,7 @@
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>validacion visual con evidencias verificables para documentar VirSem-18/VirSem-19: el mapping se inspecciona visualmente y se relaciona con clases/propiedades de la ontologia. Fixture: validation/components/semantic_virtualization/fixtures/mappings/mapping_editor_mobility_network.rml.ttl.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-07
-Marcadores visuales Playwright activos</t>
+          <t>Reconciliado 2026-05-18: SV-UI-10 está catalogado como automated/mapped y aporta evidencia visual para VirSem-18/VirSem-19 con marcadores Playwright activos.</t>
         </is>
       </c>
     </row>
@@ -14090,18 +14023,17 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>El framework queda trazado al repo oficial GTFS-Madrid-Bench antes de ejecutar una mini-fixture generada o el benchmark completo como opt-in.</t>
+          <t>El framework queda trazado al repositorio oficial GTFS-Madrid-Bench antes de derivar muestras runtime reproducibles.</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>validation/components/semantic_virtualization/gtfs_bench_official.py
-Activacion: offline/source readiness; repo local requerido</t>
+          <t>validation/components/semantic_virtualization/gtfs_bench_official.py</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: fuente oficial GTFS-Bench</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -14117,9 +14049,7 @@
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>No ejecuta el generador Docker ni valida datos generados aun. Siguiente incremento: SV-GTFS-BENCH-02 para mini-fixture derivada oficialmente.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Passed opt-in / evidencia fuente oficial generada 2026-05-07</t>
+          <t>Reconciliado 2026-05-18: valida disponibilidad local del repositorio oficial y sus mappings; no versiona un dataset reducido dentro del framework.</t>
         </is>
       </c>
     </row>
@@ -14131,7 +14061,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Generar y validar mini-fixture oficial derivada de GTFS-Madrid-Bench</t>
+          <t>Generar y validar muestra runtime derivada de GTFS-Madrid-Bench oficial</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -14151,8 +14081,8 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>- Fixture gtfs-bench-official-mini versionada en el framework
-- Repo oficial disponible solo si se desea regenerar la fixture</t>
+          <t>- Repositorio oficial GTFS-Bench sincronizado en validation/datasets/sources/gtfs-bench
+- Recursos CSV y mappings oficiales disponibles</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -14163,18 +14093,18 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>La mini-fixture oficial derivada queda validada, trazable al repo oeg-upm/gtfs-bench y lista para pruebas funcionales ligeras del virtualizador.</t>
+          <t>La muestra runtime derivada de GTFS-Bench oficial queda validada, trazable al repositorio oeg-upm/gtfs-bench y lista para pruebas funcionales ligeras del virtualizador.</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>validation/components/semantic_virtualization/gtfs_bench_mini.py
-tests/test_semantic_virtualization_gtfs_bench_mini.py</t>
+          <t>validation/components/semantic_virtualization/gtfs_bench_dataset.py
+tests/test_semantic_virtualization_gtfs_bench_dataset.py</t>
         </is>
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: muestra runtime oficial derivada</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -14191,9 +14121,7 @@
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>No sustituye el benchmark completo. El generador completo queda opt-in porque depende de servicios tipo MySQL/Docker; Level 6 conserva la ruta ligera y estable.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado / passed 2026-05-07</t>
+          <t>Reconciliado 2026-05-18: el framework no versiona un dataset reducido; deriva una muestra determinista durante la validación a partir del repositorio oficial sincronizado.</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14133,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Materializar y consultar la mini-fixture oficial derivada de GTFS-Madrid-Bench</t>
+          <t>Materializar y consultar muestra runtime derivada de GTFS-Madrid-Bench oficial</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -14225,15 +14153,15 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>- Fixture gtfs-bench-official-mini validada
-- Mapping CSV oficial disponible en references/gtfs-csv.rml.ttl
+          <t>- Muestra runtime oficial derivada validada
+- Mapping CSV oficial disponible en validation/datasets/sources/gtfs-bench/mappings/gtfs-csv.rml.ttl
 - Queries oficiales q1 disponibles</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Adaptar el mapping CSV oficial para que /data/*.csv apunte a csv/*.csv dentro de la fixture.
-Paso 2: Materializar un grafo RDF ligero desde las tablas GTFS de la mini-fixture.
+          <t>Paso 1: Adaptar el mapping CSV oficial para que /data/*.csv apunte a los CSV derivados en runtime.
+Paso 2: Materializar un grafo RDF ligero desde las tablas GTFS seleccionadas.
 Paso 3: Ejecutar la query oficial simple q1 sobre shape points.
 Paso 4: Ejecutar la query oficial completa q1 sobre shapes y shape points.
 Paso 5: Ejecutar un probe de joins ruta-viaje-parada.
@@ -14242,7 +14170,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>El mapping oficial adaptado, la mini-fixture oficial derivada y las queries oficiales producen un grafo RDF coherente y consultable.</t>
+          <t>El mapping oficial adaptado, la muestra runtime derivada y las queries oficiales producen un grafo RDF coherente y consultable.</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -14253,7 +14181,7 @@
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: materialización GTFS-Bench oficial</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -14270,9 +14198,7 @@
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>Alcance controlado: no es motor RML completo ni benchmark completo; valida coherencia funcional y consultas oficiales sobre la fixture oficial derivada sin hacer pesado Level 6.
-No computado como automatizado en 00_Resumen hasta completar la revision de la suite.
-Estado registrado previamente: Automatizado opt-in / passed 2026-05-07</t>
+          <t>Reconciliado 2026-05-18: alcance controlado y reproducible; valida coherencia funcional sobre datos derivados del repositorio oficial sin hacer pesado Level 6.</t>
         </is>
       </c>
     </row>
@@ -14294,7 +14220,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>integration / HttpData opt-in</t>
+          <t>integration / HttpData</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -14307,18 +14233,18 @@
           <t>- INESData desplegado con dos conectores
 - Semantic Virtualization desplegado
 - SV-GTFS-BENCH-03 passed
-- Ejecucion opt-in aceptada porque crea asset, policy, contract definition y negociacion</t>
+- Asset, policy, contract definition y negociación se crean con limpieza QA controlada</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Paso 1: Reutilizar la evidencia SV-GTFS-BENCH-03 para obtener gtfs_bench_official_mini_materialized.ttl.
-Paso 2: Ejecutar el runner API con --gtfs-bench-official-materialization y --skip-transfer.
+          <t>Paso 1: Reutilizar la evidencia SV-GTFS-BENCH-03 para obtener el RDF materializado derivado de GTFS-Bench oficial.
+Paso 2: Ejecutar el runner API con --gtfs-bench-official-materialization y --skip-transfer cuando se quiera acotar la validación a publicación/negociación.
 Paso 3: Verificar que el provider publica el asset HttpData con metadatos GTFS-Bench oficiales derivados.
-Paso 4: Verificar que el consumer descubre el asset en catalogo.
-Paso 5: Iniciar negociacion y esperar acuerdo FINALIZED.
-Paso 6: Ejecutar la validacion visual UI Playwright con marcadores visuales y trace desactivado.
-Paso 7: Confirmar login, detalle de catalogo, ofertas de contrato y negociacion completa.</t>
+Paso 4: Verificar que el consumer descubre el asset en catálogo.
+Paso 5: Iniciar negociación y esperar acuerdo FINALIZED.
+Paso 6: Ejecutar la validación visual UI Playwright con marcadores visuales.
+Paso 7: Confirmar login, detalle de catálogo, ofertas de contrato y negociación completa.</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -14329,14 +14255,12 @@
       <c r="I28" s="3" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/dataspace_integration.py
-validation/ui/core/07-semantic-virtualization-httpdata.spec.ts
-Activacion API: python3 validation/components/semantic_virtualization/dataspace_integration.py --gtfs-bench-official-materialization --skip-transfer
-validacion visual UI: UI_SEMANTIC_VIRTUALIZATION_HTTPDATA_DEMO=1 PLAYWRIGHT_TRACE=off</t>
+validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts</t>
         </is>
       </c>
       <c r="J28" s="12" t="inlineStr">
         <is>
-          <t>Registrado en framework / pendiente de revision de automatizacion</t>
+          <t>Automatizado / revisado: integración HttpData API+UI</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -14354,8 +14278,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>Artefactos Playwright generados localmente cuando aplica
-Resultados estructurados JSON generados por la suite</t>
+          <t>Reconciliado 2026-05-18: SV-GTFS-BENCH-04 confirma desde API y UI que el RDF oficial derivado se publica, descubre y negocia como HttpData en INESData.</t>
         </is>
       </c>
     </row>
@@ -15002,7 +14925,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>validacion visual con evidencias verificables de benchmarking: seleccion de modelos FLARES-mini, ejecucion comparativa, metricas calculadas, tabla comparativa y Best Model con elementos UI resaltados.</t>
+          <t>Validación visual con evidencias verificables de benchmarking: selección de modelos FLARES, ejecución comparativa, métricas calculadas, tabla comparativa y Best Model con elementos UI resaltados.</t>
         </is>
       </c>
     </row>
@@ -15218,7 +15141,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>validation/ui/core/10-ai-model-observer.spec.ts
+          <t>validation/ui/adapters/inesdata/specs/10-ai-model-observer.spec.ts
 validation/ui/test_cases.yaml
 validation/ui/interactive_menu.py</t>
         </is>
@@ -15511,7 +15434,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Acredita trazabilidad al repo oficial antes de generar mini-fixture oficial o benchmark completo opt-in.</t>
+          <t>Acredita trazabilidad al repositorio oficial antes de derivar muestras runtime o ejecutar validaciones pesadas fuera del ciclo habitual.</t>
         </is>
       </c>
     </row>
@@ -15539,7 +15462,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Explica que el framework usa una mini-fixture trazable al GTFS-Bench oficial sin hacer pesado Level 6.</t>
+          <t>Explica que el framework deriva una muestra runtime trazable al GTFS-Bench oficial sin hacer pesado Level 6.</t>
         </is>
       </c>
     </row>
@@ -15567,7 +15490,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Explica que la mini-fixture oficial derivada no solo existe, sino que puede convertirse a RDF y consultarse con queries oficiales.</t>
+          <t>Explica que la muestra runtime oficial derivada puede convertirse a RDF y consultarse con queries oficiales.</t>
         </is>
       </c>
     </row>
@@ -15590,7 +15513,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>SV-GTFS-BENCH-04 implementado como opt-in: el asset HttpData incluye metadatos de GTFS-Bench-official-mini, repo oficial, commit, hash del RDF, 371 triples y resultados de q1. Unit tests passed; evidencia live INESData pendiente.</t>
+          <t>SV-GTFS-BENCH-04 implementado: el asset HttpData incluye metadatos de GTFS-Bench oficial derivado, repo oficial, commit, hash del RDF, triples y resultados de consultas.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add deterministic Automap validation baseline
</commit_message>
<xml_diff>
--- a/docs/E5.2_Resultados_Validacion_Componentes.xlsx
+++ b/docs/E5.2_Resultados_Validacion_Componentes.xlsx
@@ -1370,7 +1370,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Cobertura técnica actual 20/22 (90.9%) según catálogos y suites versionadas; los pendientes quedan identificados como alcance parcial o seguimiento externo.</t>
+          <t>Cobertura técnica actual 21/23 (91.3%) según catálogos y suites versionadas; los pendientes quedan identificados como alcance parcial o seguimiento externo.</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>85/94 (90.4%) cobertura técnica trazable</t>
+          <t>86/95 (90.5%) cobertura técnica trazable</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>65/70 funcionales automatizados o revisados</t>
+          <t>66/71 funcionales automatizados o revisados</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K18" s="6" t="n">
         <v>2</v>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>16/17</t>
+          <t>17/18</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
@@ -1903,17 +1903,17 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>20/22 (90.9%)</t>
+          <t>21/23 (91.3%)</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>PT5-VS, mapping-editor, GTFS-Bench oficial e integración HttpData están implementados en el framework.</t>
+          <t>PT5-VS, mapping-editor, GTFS-Bench oficial, Automap determinista e integración HttpData están implementados en el framework.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 20 | Total: 22</t>
+          <t>Sin bloqueo: 21 | Total: 23</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>65/70</t>
+          <t>66/71</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>85/94 (90.4% cobertura técnica trazable)</t>
+          <t>86/95 (90.5% cobertura técnica trazable)</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 85 | Total: 94</t>
+          <t>Sin bloqueo: 86 | Total: 95</t>
         </is>
       </c>
       <c r="H28" s="2" t="n"/>
@@ -3426,22 +3426,22 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>PT5-VS-01..12, SV-UI-01..10, SV-GTFS-BENCH-01..04.</t>
+          <t>PT5-VS-01..12, SV-UI-01..10, SV-GTFS-BENCH-01..04 y SV-AUTOMAP-01..02.</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Ejecutar mappings offline, API SPARQL, GTFS-Bench y UI del editor desde nivel 6.</t>
+          <t>Ejecutar mappings offline, API SPARQL, GTFS-Bench, Automap determinista y UI del editor desde nivel 6.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Implementado técnicamente / 20 de 22 casos trazados</t>
+          <t>Implementado técnicamente / 21 de 23 casos trazados</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Cobertura técnica real 20/22 (90.9%); progreso operativo registrado como 10/22 (45.5%) hasta que QA valide manualmente los tests del Virtualizador.</t>
+          <t>Cobertura técnica real 21/23 (91.3%) con Automap fase 2 determinista incluida; quedan pendientes la integración específica con Ontology Hub y la revisión final de Level 6 sin Kafka.</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>DS-UI-SV-01 y SV-GTFS-BENCH-04 están automatizados; para el cierre operativo se computa solo la mitad del avance real hasta revisión QA.</t>
+          <t>DS-UI-SV-01 y SV-GTFS-BENCH-04 están automatizados; el avance debe computarse con resultados reales de ejecución y no con descuentos temporales.</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>Conservar evidencia actual y validar resultados antes de contabilizar el 100% técnico del Virtualizador.</t>
+          <t>Conservar evidencia actual, reejecutar Level 6 sin Kafka y documentar fallos reales si aparecen.</t>
         </is>
       </c>
     </row>
@@ -12729,7 +12729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="53" customWidth="1" style="26" min="1" max="1"/>
@@ -13707,12 +13707,13 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>validation/components/semantic_virtualization/mapping_validation.py</t>
+          <t>validation/components/semantic_virtualization/mapping_validation.py
+validation/components/semantic_virtualization/automap_execution.py</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Automatizado / revisado: evaluación de métodos</t>
+          <t>Automatizado / revisado: evaluación de métodos + Automap determinista</t>
         </is>
       </c>
       <c r="K16" s="9" t="inlineStr">
@@ -13729,43 +13730,120 @@
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; la suite compara métodos con criterios reproducibles.</t>
+          <t>PT5-VS-10 queda respaldado por la comparación de métodos offline y por SV-AUTOMAP-02 como baseline determinista de Automap sin LLM.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1" s="26">
       <c r="A17" s="9" t="inlineStr">
         <is>
+          <t>SV-AUTOMAP-02</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Línea base determinista de Automap para generación y evaluación de mappings</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Semantic Virtualization</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>functional / mapping generation</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>QA / Semantic Engineer</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>- Repositorio Automap sincronizado por Level 5
+- Fixtures versionados de movilidad disponibles
+- No se requieren claves LLM ni .env</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Validar que el checkout local de Automap está disponible.
+Paso 2: Cargar fixture CSV de movilidad y extraer esquema con las utilidades de Automap.
+Paso 3: Extraer contexto de ontología desde el fixture Turtle.
+Paso 4: Materializar RDF controlado y ejecutar una consulta ASK.
+Paso 5: Comparar el KG generado contra un gold KG mediante las métricas de Automap.</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Automap deterministic tooling extracts schema and ontology context, produces RDF evidence and matches the gold KG metrics.</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/semantic_virtualization/automap_execution.py
+tests/test_semantic_virtualization_automap_execution.py</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Automatizado / revisado: baseline determinista Automap</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite
+KG RDF generado y métricas comparadas contra gold KG</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>Repositorio Automap
+Entregable técnico de Semantic Virtualization</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Trazado a PT5-VS-01, PT5-VS-06 y PT5-VS-10. No ejecuta LLM en Level 6 para evitar dependencias de secretos/modelos externos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" s="26">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
           <t>PT5-VS-11</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Desplegar motor y acceder vía conector INESData</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>integration</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>- Conectores provider/consumer de INESData accesibles
 - Endpoint HttpData del virtualizador alcanzable desde los pods del conector</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Provider registra como asset HttpData la salida o endpoint del virtualizador.
 Paso 2: Consumer abre el catálogo de INESData.
@@ -13774,23 +13852,23 @@
 Paso 5: Verificar que el asset queda accesible bajo gobierno del conector.</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>The virtualized output is exposed as HttpData and negotiable from INESData</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr">
         <is>
           <t>validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts
 validation/components/semantic_virtualization/dataspace_integration.py</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: integración INESData HttpData</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K18" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright generados localmente cuando aplica
@@ -13798,51 +13876,51 @@
 Dashboard local de experimento generado por el framework</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: DS-UI-SV-01 confirma desde UI de INESData que el motor virtualizado se publica como HttpData, se descubre y se negocia. La ruta Playwright actual es validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1" s="26">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" ht="48" customHeight="1" s="26">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>PT5-VS-12</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Provocar errores controlados en consultas o mappings</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>functional</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>- Endpoint SPARQL accesible
 - Consulta inválida controlada preparada por la suite</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Enviar una consulta SPARQL inválida o un mapping inválido controlado.
 Paso 2: Esperar respuesta del servicio o validador.
@@ -13850,72 +13928,72 @@
 Paso 4: Guardar el diagnóstico como evidencia.</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Invalid SPARQL input returns a controlled HTTP 4xx diagnostic response</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I19" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/runner.py</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>Automatizado / revisado: errores controlados</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L18" s="9" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M18" s="9" t="inlineStr">
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: el catálogo YAML marca coverage_status=automated y mapping_status=mapped; runner.py valida respuesta HTTP 4xx controlada ante consulta inválida.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1" s="26">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="20" ht="48" customHeight="1" s="26">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>SV-UI-04</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Explorar paneles de ontologías en el mapping-editor</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al URL del mapping-editor.
 Paso 2: Click en "Ontologies" en el menu lateral.
@@ -13923,73 +14001,73 @@
 Paso 4: Capturar evidencia visual y JSON del estado.</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>La UI muestra el flujo de carga, exploracion y visualizacion de ontologías documentado en E3.1.</t>
         </is>
       </c>
-      <c r="I19" s="9" t="inlineStr">
+      <c r="I20" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: paneles de ontologías visibles</t>
         </is>
       </c>
-      <c r="K19" s="9" t="inlineStr">
+      <c r="K20" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite
 Dashboard local de experimento generado por el framework</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr">
+      <c r="L20" s="9" t="inlineStr">
         <is>
           <t>Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M19" s="9" t="inlineStr">
+      <c r="M20" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-06/PT5-VS-07; evidencia previa con marcadores visuales Playwright.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" s="26">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21" ht="48" customHeight="1" s="26">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>SV-UI-05</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Crear mapping temporal y abrir authoring de TriplesMap</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor habilitado por la validación del componente
 - Sesión Streamlit nueva para la prueba</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al mapping-editor.
 Paso 2: Click en "Global Configuration".
@@ -13999,73 +14077,73 @@
 Paso 6: Verificar entrada "Add TriplesMap" o mensaje controlado de precondicion por falta de fuentes de datos.</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>La UI permite iniciar un mapping y entrar al flujo de construccion sin crear recursos en el conector ni en Kubernetes.</t>
         </is>
       </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="I21" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: authoring no destructivo</t>
         </is>
       </c>
-      <c r="K20" s="9" t="inlineStr">
+      <c r="K21" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite
 Dashboard local de experimento generado por el framework</t>
         </is>
       </c>
-      <c r="L20" s="9" t="inlineStr">
+      <c r="L21" s="9" t="inlineStr">
         <is>
           <t>Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M20" s="9" t="inlineStr">
+      <c r="M21" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-01, PT5-VS-05 y PT5-VS-06; la mutación queda limitada a la sesión del navegador.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1" s="26">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22" ht="48" customHeight="1" s="26">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>SV-UI-06</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Revisar checkpoints de exportacion y materializacion</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor habilitado por la validación del componente
 - Mapping temporal creado en sesión</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al mapping-editor.
 Paso 2: Crear un mapping temporal desde "Global Configuration".
@@ -14075,74 +14153,74 @@
 Paso 6: Capturar ambas pantallas.</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>La UI expone checkpoints de exportacion de mappings y materializacion de grafos, con precondiciones controladas.</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: exportacion/materializacion visibles</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K22" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite
 Dashboard local de experimento generado por el framework</t>
         </is>
       </c>
-      <c r="L21" s="9" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M21" s="9" t="inlineStr">
+      <c r="M22" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: flujo UI automatizado como soporte funcional de PT5-VS-08 y PT5-VS-09; no requiere ejecutar Morph-KGC si no hay fuentes configuradas.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1" s="26">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="23" ht="48" customHeight="1" s="26">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>SV-UI-07</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Configurar namespace y exportar mapping desde el editor</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible
 - Sesión Streamlit nueva para la prueba</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al URL del mapping-editor.
 Paso 2: Abrir Global Configuration.
@@ -14155,74 +14233,74 @@
 Paso 9: Abrir Set Style para capturar evidencia visual de controles de estilo.</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>La UI permite crear un mapping temporal, asociar un namespace custom, exponer la exportacion del mapping y mostrar controles de estilo sin mutar INESData ni Kubernetes.</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: namespace y exportación desde editor</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="K23" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L22" s="9" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M22" s="9" t="inlineStr">
+      <c r="M23" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: SV-UI-07 está catalogado como automated/mapped y la evidencia visual se generó en 2026-05-07; Level 6 lo incorpora dentro de la suite UI del componente.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1" s="26">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="24" ht="48" customHeight="1" s="26">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>SV-UI-08</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Importar ontología y fuente CSV desde el mapping-editor</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor habilitado por la validación del componente
 - UI del editor accesible
 - Fixtures de ontología y CSV disponibles en el framework</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al URL del mapping-editor.
 Paso 2: Abrir Global Configuration.
@@ -14236,74 +14314,74 @@
 Paso 10: Abrir Display Data para confirmar que la fuente queda disponible.</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>La UI importa una ontología fixture, permite explorar sus términos, carga una fuente CSV fixture y deja ambos insumos disponibles para flujos posteriores de authoring de mappings.</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: importación de ontología y CSV</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
+      <c r="K24" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L23" s="9" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M23" s="9" t="inlineStr">
+      <c r="M24" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: SV-UI-08 está catalogado como automated/mapped; usa fixtures controlados del componente para validar la UI sin versionar datasets reducidos de dominio.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1" s="26">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="25" ht="48" customHeight="1" s="26">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>SV-UI-10</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Explorar mapping no vacio y Ontology-Mapping Lens</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>functional UI validación visual</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>- mapping-editor desplegado y accesible
 - Fixture RML no vacía compatible con el editor
 - Ontología de movilidad controlada disponible</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ingresar al URL del mapping-editor.
 Paso 2: Click en "Global Configuration".
@@ -14319,216 +14397,216 @@
 Paso 12: Revisar "Mapping Composition", "Class Usage", "Property Usage" y "External Terms".</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>La UI importa un mapping RML no vacio, muestra su red visual, búsquedas predefinidas, preview y paneles de explicabilidad del lens.</t>
         </is>
       </c>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/ui/specs/sv_ui_02_mapping_editor.spec.js
 Variable runtime: SEMANTIC_VIRTUALIZATION_MAPPING_EDITOR_UI=1
 Marcadores: PLAYWRIGHT_INTERACTION_MARKERS=1</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: mapping no vacío y Ontology-Mapping Lens</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr">
+      <c r="K25" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L24" s="9" t="inlineStr">
+      <c r="L25" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M24" s="9" t="inlineStr">
+      <c r="M25" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: SV-UI-10 está catalogado como automated/mapped y aporta evidencia visual para VirSem-18/VirSem-19 con marcadores Playwright activos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1" s="26">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>SV-GTFS-BENCH-01</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Validar recursos oficiales GTFS-Madrid-Bench para virtualizacion</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Semantic Virtualization</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>support / official dataset traceability</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>QA / Data Space Operator</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>Repositorio fuente del componente integrado en el entorno</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework</t>
-        </is>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>El framework queda trazado al repositorio oficial GTFS-Madrid-Bench antes de derivar muestras reproducibles.</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>validation/components/semantic_virtualization/gtfs_bench_official.py</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Automatizado / revisado: fuente oficial GTFS-Bench</t>
-        </is>
-      </c>
-      <c r="K25" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework de validación
-Resultados estructurados JSON generados por la suite</t>
-        </is>
-      </c>
-      <c r="L25" s="9" t="inlineStr">
-        <is>
-          <t>Entregable E5.1 de validación</t>
-        </is>
-      </c>
-      <c r="M25" s="9" t="inlineStr">
-        <is>
-          <t>Reconciliado 2026-05-18: valida disponibilidad local del repositorio oficial y sus mappings; no versiona un dataset reducido dentro del framework.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1" s="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
+          <t>SV-GTFS-BENCH-01</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Validar recursos oficiales GTFS-Madrid-Bench para virtualizacion</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Semantic Virtualization</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>support / official dataset traceability</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>QA / Data Space Operator</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Repositorio fuente del componente integrado en el entorno</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>El framework queda trazado al repositorio oficial GTFS-Madrid-Bench antes de derivar muestras reproducibles.</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/semantic_virtualization/gtfs_bench_official.py</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Automatizado / revisado: fuente oficial GTFS-Bench</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>Entregable E5.1 de validación</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>Reconciliado 2026-05-18: valida disponibilidad local del repositorio oficial y sus mappings; no versiona un dataset reducido dentro del framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" s="26">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
           <t>SV-GTFS-BENCH-02</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Generar y validar muestra derivada de GTFS-Madrid-Bench oficial</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>support / trazabilidad dataset oficial</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>QA / Validación</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>- Repositorio oficial GTFS-Bench sincronizado por el framework
 - Recursos CSV y mappings oficiales disponibles como insumo reproducible</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>La muestra derivada de GTFS-Bench oficial queda validada, trazable al repositorio oeg-upm/gtfs-bench y lista para pruebas funcionales ligeras del virtualizador.</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="I27" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/gtfs_bench_dataset.py
 tests/test_semantic_virtualization_gtfs_bench_dataset.py</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: muestra oficial derivada</t>
         </is>
       </c>
-      <c r="K26" s="9" t="inlineStr">
+      <c r="K27" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L26" s="9" t="inlineStr">
+      <c r="L27" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M26" s="9" t="inlineStr">
+      <c r="M27" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: el framework no versiona un dataset reducido; deriva una muestra determinista durante la validación a partir del repositorio oficial sincronizado.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="48" customHeight="1" s="26">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28" ht="48" customHeight="1" s="26">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>SV-GTFS-BENCH-03</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Materializar y consultar muestra derivada de GTFS-Madrid-Bench oficial</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>functional / trazabilidad dataset oficial</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>QA / Validación</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>- Muestra oficial derivada validada
 - Mapping CSV oficial disponible como insumo reproducible
 - Queries oficiales q1 disponibles</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Adaptar el mapping CSV oficial para apuntar a los CSV derivados para la validación.
 Paso 2: Materializar un grafo RDF ligero desde las tablas GTFS seleccionadas.
@@ -14537,67 +14615,67 @@
 Paso 5: Registrar estadísticas RDF y resultados SPARQL.</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t>El mapping oficial adaptado, la muestra derivada y las queries oficiales producen un grafo RDF coherente y consultable.</t>
         </is>
       </c>
-      <c r="I27" s="9" t="inlineStr">
+      <c r="I28" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/gtfs_bench_materialization.py
 tests/test_semantic_virtualization_gtfs_bench_materialization.py</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: materialización GTFS-Bench oficial</t>
         </is>
       </c>
-      <c r="K27" s="9" t="inlineStr">
+      <c r="K28" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L27" s="9" t="inlineStr">
+      <c r="L28" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M27" s="9" t="inlineStr">
+      <c r="M28" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: alcance controlado y reproducible; valida coherencia funcional sobre datos derivados del repositorio oficial sin hacer pesado Level 6.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1" s="26">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29" ht="135" customHeight="1" s="26">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>SV-GTFS-BENCH-04</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Exponer RDF oficial derivado de GTFS-Bench como asset HttpData en INESData</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization + INESData</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>integration / HttpData</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>Provider / Consumer / QA / Validación</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>- INESData desplegado con dos conectores
 - Semantic Virtualization desplegado
@@ -14605,7 +14683,7 @@
 - Asset, policy, contract definition y negociación se crean con limpieza QA controlada</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Reutilizar la evidencia SV-GTFS-BENCH-03 para obtener el RDF materializado derivado de GTFS-Bench oficial.
 Paso 2: Ejecutar el runner API con --gtfs-bench-official-materialization y --skip-transfer cuando se quiera acotar la validación a publicación/negociación.
@@ -14616,75 +14694,75 @@
 Paso 7: Confirmar login, detalle de catálogo, ofertas de contrato y negociación completa.</t>
         </is>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t>El RDF oficial derivado del virtualizador queda registrado como asset HttpData gobernado por INESData, descubrible y negociable por el consumer desde API y UI.</t>
         </is>
       </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="I29" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/dataspace_integration.py
 validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Automatizado / revisado: integración HttpData API+UI</t>
         </is>
       </c>
-      <c r="K28" s="9" t="inlineStr">
+      <c r="K29" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L28" s="9" t="inlineStr">
+      <c r="L29" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Semantic Virtualization</t>
         </is>
       </c>
-      <c r="M28" s="9" t="inlineStr">
+      <c r="M29" s="9" t="inlineStr">
         <is>
           <t>Reconciliado 2026-05-18: SV-GTFS-BENCH-04 confirma desde API y UI que el RDF oficial derivado se publica, descubre y negocia como HttpData en INESData.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="135" customHeight="1" s="26">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="30" ht="90" customHeight="1" s="26">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>INT-VS-DS-01</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Publicación HttpData del virtualizador en INESData</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization + INESData</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>integration</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>Data Provider / Data Consumer / QA</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>- Virtualizador desplegado
 - Conectores INESData operativos
 - Endpoint de consulta/salida semántica disponible</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Crear asset HttpData hacia el virtualizador.
 Paso 2: Crear policy y contract definition.
@@ -14692,74 +14770,74 @@
 Paso 4: Registrar trazabilidad de asset/acuerdo.</t>
         </is>
       </c>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>El output del virtualizador queda gobernado como asset de dataspace.</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr">
+      <c r="I30" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/dataspace_integration.py</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Automatizado / mapped / Level 6 por defecto</t>
         </is>
       </c>
-      <c r="K29" s="9" t="inlineStr">
+      <c r="K30" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright/JSON generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L29" s="9" t="inlineStr">
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico del componente
 Catálogos YAML del framework</t>
         </is>
       </c>
-      <c r="M29" s="9" t="inlineStr">
+      <c r="M30" s="9" t="inlineStr">
         <is>
           <t>Relacionado con PT5-VS-11 y DS-UI-SV-01.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="90" customHeight="1" s="26">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="31" ht="75" customHeight="1" s="26">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>INT-VS-DS-02</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Negociación visual del asset semántico desde INESData UI</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization + INESData</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>integration UI</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E31" s="9" t="inlineStr">
         <is>
           <t>Data Consumer / QA</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>- Asset HttpData semántico visible
 - Consumer puede acceder a Catalog Browser</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Abrir Catalog Browser.
 Paso 2: Localizar asset semántico.
@@ -14767,257 +14845,257 @@
 Paso 4: Negociar contrato desde la UI.</t>
         </is>
       </c>
-      <c r="H30" s="9" t="inlineStr">
+      <c r="H31" s="9" t="inlineStr">
         <is>
           <t>La negociación visual del asset semántico queda evidenciada con Playwright.</t>
         </is>
       </c>
-      <c r="I30" s="9" t="inlineStr">
+      <c r="I31" s="9" t="inlineStr">
         <is>
           <t>validation/ui/adapters/inesdata/specs/07-semantic-virtualization-httpdata.spec.ts</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>Automatizado / mapped / Level 6 dataspace</t>
         </is>
       </c>
-      <c r="K30" s="9" t="inlineStr">
+      <c r="K31" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright/JSON generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L30" s="9" t="inlineStr">
+      <c r="L31" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico del componente
 Catálogos YAML del framework</t>
         </is>
       </c>
-      <c r="M30" s="9" t="inlineStr">
+      <c r="M31" s="9" t="inlineStr">
         <is>
           <t>Nivel 6 incluye la spec 07 por defecto.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="75" customHeight="1" s="26">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="32" ht="135" customHeight="1" s="26">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>INT-VS-AMH-01</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Salida virtualizada trazable hacia AI Model Hub</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization + AI Model Hub</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>integration traceability</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>QA / Auditoría</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>- Muestra GTFS-Bench oficial derivada
 - Caso MH-MOB-01 disponible</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Validar materialización GTFS-Bench.
 Paso 2: Comparar hashes, filas y join keys.
 Paso 3: Registrar puente con AI Model Hub movilidad.</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="H32" s="9" t="inlineStr">
         <is>
           <t>La salida semántica tiene trazabilidad defendible hacia el caso de movilidad de AI Model Hub.</t>
         </is>
       </c>
-      <c r="I31" s="9" t="inlineStr">
+      <c r="I32" s="9" t="inlineStr">
         <is>
           <t>validation/components/ai_model_hub/virtualization_traceability.py</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>Automatizado / mapped / Level 6 por defecto</t>
         </is>
       </c>
-      <c r="K31" s="9" t="inlineStr">
+      <c r="K32" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Artefactos Playwright/JSON generados localmente cuando aplica
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L31" s="9" t="inlineStr">
+      <c r="L32" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico del componente
 Catálogos YAML del framework</t>
         </is>
       </c>
-      <c r="M31" s="9" t="inlineStr">
+      <c r="M32" s="9" t="inlineStr">
         <is>
           <t>No implica consumo directo en UI de AI Model Hub todavía; funciona como puente de trazabilidad.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="135" customHeight="1" s="26">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="33" ht="100.8" customHeight="1" s="26">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>INT-VS-OH-01</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Alineación Virtualización con ontologías de Ontology Hub</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization + Ontology Hub</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>integration</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>Semantic Engineer / QA</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>- Ontologías de referencia disponibles en Ontology Hub
 - Mapping del virtualizador declarando dependencia semántica</t>
         </is>
       </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Identificar ontología de referencia.
 Paso 2: Asociarla al mapping o fixture.
 Paso 3: Validar que la integración queda evidenciada en resultados.</t>
         </is>
       </c>
-      <c r="H32" s="9" t="inlineStr">
+      <c r="H33" s="9" t="inlineStr">
         <is>
           <t>El mapping del virtualizador declara y usa una referencia de Ontology Hub de forma verificable.</t>
         </is>
       </c>
-      <c r="I32" s="9" t="inlineStr">
+      <c r="I33" s="9" t="inlineStr">
         <is>
           <t>Pendiente de automatización específica</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>Pendiente / partial</t>
         </is>
       </c>
-      <c r="K32" s="9" t="inlineStr">
+      <c r="K33" s="9" t="inlineStr">
         <is>
           <t>Pendiente de evidencia final</t>
         </is>
       </c>
-      <c r="L32" s="9" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico del componente
 Catálogos YAML del framework</t>
         </is>
       </c>
-      <c r="M32" s="9" t="inlineStr">
+      <c r="M33" s="9" t="inlineStr">
         <is>
           <t>Único caso de integración del virtualizador marcado como partial en el catálogo YAML actual.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="100.8" customHeight="1" s="26">
-      <c r="A33" s="9" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>SV-COVERAGE-SNAPSHOT</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Cobertura técnica vigente del Virtualizador</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Semantic Virtualization</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>governance / cierre A5.2</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E34" s="9" t="inlineStr">
         <is>
           <t>QA / Validación</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>- Suites del Virtualizador versionadas
 - Catálogos actualizados con el estado real del framework</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
         <is>
           <t>Paso 1: Ejecutar Level 6.
 Paso 2: Revisar dashboard y artefactos generados.
 Paso 3: Registrar incidencias reales del componente o del framework.</t>
         </is>
       </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>El workbook refleja 20/22 (90.9%) como avance técnico vigente del Virtualizador.</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="inlineStr">
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>El workbook refleja 21/23 (91.3%) como avance técnico vigente del Virtualizador.</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/test_cases.yaml
 validation/projects/inesdata/integration/test_cases.yaml</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Estado real registrado</t>
-        </is>
-      </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Estado real registrado con Automap fase 2 determinista</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L33" s="9" t="inlineStr">
+      <c r="L34" s="9" t="inlineStr">
         <is>
           <t>Catálogos YAML del framework
 E5.2 cierre A5.2</t>
         </is>
       </c>
-      <c r="M33" s="9" t="inlineStr">
-        <is>
-          <t>Sustituye la lectura temporal previa; la vista ejecutiva ya refleja la cobertura técnica vigente.</t>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>Pendientes principales: integración específica con Ontology Hub y revisión final de ejecución Level 6 sin Kafka.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update A5.2 traceability for Automap reuse
</commit_message>
<xml_diff>
--- a/docs/E5.2_Resultados_Validacion_Componentes.xlsx
+++ b/docs/E5.2_Resultados_Validacion_Componentes.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_Trazabilidad_OH'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_Estado_Cobertura'!$A$1:$J$16</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>86/95 (90.5%) cobertura técnica trazable</t>
+          <t>87/95 (91.6%) cobertura técnica trazable</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>20/24 integraciones automatizadas o revisadas</t>
+          <t>21/24 integraciones automatizadas o revisadas</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Incluye integración INESData/HttpData y suites API/UI. Kafka se valida aparte por activación explícita.</t>
+          <t>Incluye integración INESData/HttpData, reutilización Ontology Hub/Automap y suites API/UI. Kafka se valida aparte por activación explícita.</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -1895,25 +1895,25 @@
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>21/23 (91.3%)</t>
+          <t>22/23 (95.7%)</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>PT5-VS, mapping-editor, GTFS-Bench oficial, Automap determinista e integración HttpData están implementados en el framework.</t>
+          <t>PT5-VS, mapping-editor, GTFS-Bench oficial, Automap determinista, reutilización Ontology Hub e integración HttpData están implementados en el framework.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 21 | Total: 23</t>
+          <t>Sin bloqueo: 22 | Total: 23</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="D28" s="7">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>86/95 (90.5% cobertura técnica trazable)</t>
+          <t>87/95 (91.6% cobertura técnica trazable)</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 86 | Total: 95</t>
+          <t>Sin bloqueo: 87 | Total: 95</t>
         </is>
       </c>
       <c r="H28" s="2" t="n"/>
@@ -3436,12 +3436,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Implementado técnicamente / 21 de 23 casos trazados</t>
+          <t>Implementado técnicamente / 22 de 23 casos trazados</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Cobertura técnica real 21/23 (91.3%) con Automap fase 2 determinista incluida; quedan pendientes la integración específica con Ontology Hub y la revisión final de Level 6 sin Kafka.</t>
+          <t>Cobertura técnica real 22/23 (95.7%) con Automap fase 2 determinista y reutilización Ontology Hub incluidas; queda pendiente la revisión final de Level 6 sin Kafka y el registro de incidencias reales si aparecen.</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>La integración explícita con Ontology Hub sigue parcial y, además, la revisión QA del conjunto del Virtualizador está pendiente.</t>
+          <t>La integración explícita con Ontology Hub queda cubierta por mapping_validation y automap_execution. La revisión QA del conjunto del Virtualizador sigue pendiente de la ejecución final.</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Línea base determinista de Automap para generación y evaluación de mappings</t>
+          <t>Línea base determinista de Automap para generación, evaluación y reutilización semántica</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>functional / mapping generation</t>
+          <t>functional / mapping generation / semantic reuse</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -13764,6 +13764,7 @@
         <is>
           <t>- Repositorio Automap sincronizado por Level 5
 - Fixtures versionados de movilidad disponibles
+- Ontología de referencia gobernable por Ontology Hub disponible
 - No se requieren claves LLM ni .env</t>
         </is>
       </c>
@@ -13771,38 +13772,40 @@
         <is>
           <t>Paso 1: Validar que el checkout local de Automap está disponible.
 Paso 2: Cargar fixture CSV de movilidad y extraer esquema con las utilidades de Automap.
-Paso 3: Extraer contexto de ontología desde el fixture Turtle.
-Paso 4: Materializar RDF controlado y ejecutar una consulta ASK.
-Paso 5: Comparar el KG generado contra un gold KG mediante las métricas de Automap.</t>
+Paso 3: Extraer contexto de ontología desde el fixture Turtle propio y desde el artefacto gobernable por Ontology Hub.
+Paso 4: Materializar RDF controlado con ambos conjuntos de términos y ejecutar consultas ASK.
+Paso 5: Comparar los KGs generados contra gold KGs mediante las métricas de Automap.</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Automap deterministic tooling extracts schema and ontology context, produces RDF evidence and matches the gold KG metrics.</t>
+          <t>Automap deterministic tooling extracts schema and ontology context, reuses an Ontology Hub-governable ontology artifact, produces RDF evidence and matches the gold KG metrics.</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
           <t>validation/components/semantic_virtualization/automap_execution.py
-tests/test_semantic_virtualization_automap_execution.py</t>
+tests/test_semantic_virtualization_automap_execution.py
+validation/components/semantic_virtualization/fixtures/ontology/mobility-mini.ttl</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Automatizado / revisado: baseline determinista Automap</t>
+          <t>Automatizado / revisado: baseline determinista Automap + reutilización Ontology Hub</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite
-KG RDF generado y métricas comparadas contra gold KG</t>
+KGs RDF generados y métricas comparadas contra gold KGs</t>
         </is>
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
           <t>Repositorio Automap
-Entregable técnico de Semantic Virtualization</t>
+Entregable técnico de Semantic Virtualization
+Artefactos de referencia de Ontology Hub</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -14982,35 +14985,41 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>- Ontologías de referencia disponibles en Ontology Hub
-- Mapping del virtualizador declarando dependencia semántica</t>
+          <t>- Ontología de referencia gobernable por Ontology Hub disponible como Turtle/RDF
+- Mapping del virtualizador declarando dependencia semántica
+- Baseline Automap reutilizando los términos de esa ontología</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>Paso 1: Identificar ontología de referencia.
-Paso 2: Asociarla al mapping o fixture.
-Paso 3: Validar que la integración queda evidenciada en resultados.</t>
+          <t>Paso 1: Identificar ontología de referencia con metadatos OWL/RDFS.
+Paso 2: Asociarla al mapping o fixture del virtualizador.
+Paso 3: Ejecutar validación offline de mapeo y baseline Automap con los términos de la ontología.
+Paso 4: Validar que la integración queda evidenciada en resultados estructurados.</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>El mapping del virtualizador declara y usa una referencia de Ontology Hub de forma verificable.</t>
+          <t>El mapping del virtualizador y la baseline Automap reutilizan una referencia de Ontology Hub de forma verificable.</t>
         </is>
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>Pendiente de automatización específica</t>
+          <t>validation/components/semantic_virtualization/mapping_validation.py
+validation/components/semantic_virtualization/automap_execution.py
+validation/components/semantic_virtualization/fixtures/ontology/mobility-mini.ttl</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Pendiente / partial</t>
+          <t>Automatizado / revisado</t>
         </is>
       </c>
       <c r="K33" s="9" t="inlineStr">
         <is>
-          <t>Pendiente de evidencia final</t>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por mapping_validation y automap_execution
+KG RDF generado con términos gobernables por Ontology Hub</t>
         </is>
       </c>
       <c r="L33" s="9" t="inlineStr">
@@ -15067,7 +15076,7 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>El workbook refleja 21/23 (91.3%) como avance técnico vigente del Virtualizador.</t>
+          <t>El workbook refleja 22/23 (95.7%) como avance técnico vigente del Virtualizador.</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr">
@@ -15078,7 +15087,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Estado real registrado con Automap fase 2 determinista</t>
+          <t>Estado real registrado con Automap fase 2 determinista y reutilización Ontology Hub</t>
         </is>
       </c>
       <c r="K34" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Update A5.2 closure evidence after Level 6
</commit_message>
<xml_diff>
--- a/docs/E5.2_Resultados_Validacion_Componentes.xlsx
+++ b/docs/E5.2_Resultados_Validacion_Componentes.xlsx
@@ -1323,7 +1323,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Automatizado alto / pendiente evidencia final de cierre</t>
+          <t>Automatizado con baseline controlada / pendiente evidencia final sin Kafka</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Último Level 6 disponible: AI Model Hub 27/27 passed. Persisten como dependencia de cierre los modelos reales GTFS/FLARES y la evidencia final sin Kafka.</t>
+          <t>Último Level 6 disponible: AI Model Hub 27/27 passed. La baseline A5.2 usa model-server controlado para FLARES/GTFS; los modelos reales quedan como reemplazo/evolución del componente, no como bloqueo del framework.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Cobertura técnica actual 21/23 (91.3%) según catálogos y suites versionadas; los pendientes quedan identificados como alcance parcial o seguimiento externo.</t>
+          <t>Cobertura técnica actual 22/23 (95.7%) según catálogos y suites versionadas; queda revisión final de Level 6 sin Kafka y seguimiento de incidencias reales si aparecen.</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>87/95 (91.6%) cobertura técnica trazable</t>
+          <t>92/95 (96.8%) cobertura técnica trazable</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>21/24 integraciones automatizadas o revisadas</t>
+          <t>23/24 integraciones automatizadas o revisadas</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Incluye integración INESData/HttpData, reutilización Ontology Hub/Automap y suites API/UI. Kafka se valida aparte por activación explícita.</t>
+          <t>Incluye integración INESData/HttpData, AI Model Hub con Observer, reutilización Ontology Hub/Automap y suites API/UI. Kafka se valida aparte por activación explícita.</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J17" s="6" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
@@ -1625,12 +1625,12 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Level 6 final sin Kafka, ejecución Kafka explícita de cierre y seguimiento de incidencias conocidas de componentes</t>
+          <t>Level 6 sin Kafka ejecutado con fallos conocidos de Ontology Hub; queda ejecución Kafka explícita</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Pendientes no asociados a descuento técnico; reflejan fallos/dependencias externas, alcance parcial o suites explícitas por coste temporal.</t>
+          <t>El experimento 2026-05-22_09-38-34 valida AI Model Hub y Semantic Virtualization. Los pendientes vigentes se concentran en Ontology Hub: OH-APP-10, OH-APP-22 y PT5-OH-13.</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -1644,10 +1644,10 @@
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Integración PT5 y baseline funcional; incidencias conocidas siguen documentadas.</t>
+          <t>Integración PT5 y baseline funcional ejecutadas; persisten OH-APP-10, OH-APP-22 y PT5-OH-13 como incidencias del componente.</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1849,30 +1849,30 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>12/12</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>28/32 (87.5%)</t>
+          <t>32/32 (100.0%)</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Observer MH-OBS-01/MH-OBS-02 queda automatizado y mapeado; MH-OBS-03..06 siguen planificados.</t>
+          <t>PT5-MH, FLARES, GTFS, DAIMO, Observer y flujos INESData quedan automatizados con baseline controlada; los modelos reales son reemplazables cuando estén disponibles.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 28 | Total: 32</t>
+          <t>Sin bloqueo: 32 | Total: 32</t>
         </is>
       </c>
       <c r="H26" s="2" t="n"/>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>17/18</t>
+          <t>18/18</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
@@ -1899,21 +1899,21 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>22/23 (95.7%)</t>
+          <t>23/23 (100.0%)</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>PT5-VS, mapping-editor, GTFS-Bench oficial, Automap determinista, reutilización Ontology Hub e integración HttpData están implementados en el framework.</t>
+          <t>PT5-VS, mapping-editor, GTFS-Bench oficial, Automap determinista, reutilización Ontology Hub e integración HttpData pasaron en Level 6 2026-05-22.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 22 | Total: 23</t>
+          <t>Sin bloqueo: 23 | Total: 23</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>66/71</t>
+          <t>69/71</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="D28" s="7">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>87/95 (91.6% cobertura técnica trazable)</t>
+          <t>92/95 (96.8% cobertura técnica trazable)</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Sin bloqueo: 87 | Total: 95</t>
+          <t>Sin bloqueo: 92 | Total: 95</t>
         </is>
       </c>
       <c r="H28" s="2" t="n"/>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
+          <t>Level 6 2026-05-22: passed</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Mantener como issue/cobertura pendiente de componente y reejecutar después de corrección.</t>
+          <t>Cerrado en la ejecución 2026-05-22; no mantener como pendiente vigente.</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
+          <t>Level 6 2026-05-22: passed</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Reportar/actualizar issue versions.js ENOENT y reejecutar después de corrección.</t>
+          <t>Cerrado en la ejecución 2026-05-22; el bloque de versiones pasó.</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
+          <t>Level 6 2026-05-22: passed</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Mantener como issue/cobertura pendiente de componente y reejecutar después de corrección.</t>
+          <t>Cerrado en la ejecución 2026-05-22; detalle y descarga .n3 pasaron.</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Baseline idempotente marcada 2026-05-07: skipped</t>
+          <t>Level 6 2026-05-22: failed HTTP 502</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Mantener como issue/cobertura pendiente de componente y reejecutar después de corrección.</t>
+          <t>Mantener como incidencia vigente del componente: endpoint SPARQL público devuelve 502 en pt5_oh_13_sparql_access.</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -3222,12 +3222,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Casi cerrado: baseline funcional 2026-05-07 19:27:24 ejecutada con 25/27 passed</t>
+          <t>Casi cerrado: Level 6 2026-05-22 con 25/27 funcionales y 4/5 integración</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>La suite funcional completa pasa 25/27. OH-APP-05, OH-APP-12, OH-APP-13, OH-APP-15 y OH-APP-17 quedan recuperados. Persisten OH-APP-10 y OH-APP-22 como issues de componente; versionado ENOENT queda abierto aúnque el framework tolere la recuperación.</t>
+          <t>La suite funcional completa pasa 25/27. OH-APP-17, bloque de versiones, ficha .n3, FOOPS y Themis pasan. Persisten OH-APP-10 y OH-APP-22; integración SPARQL PT5-OH-13 devuelve HTTP 502.</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
@@ -3240,12 +3240,12 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Persisten fallos de componente: OH-APP-10 metadata/tags no se publican tras Save; OH-APP-22 Patterns devuelve 500; versions.js ENOENT aún puede reiniciar el pod aúnque la suite se recupere.</t>
+          <t>Persisten fallos de componente: OH-APP-10 metadata/tags no se publican tras Save; OH-APP-22 Patterns devuelve 500; PT5-OH-13 SPARQL devuelve 502.</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>Actualizar issues de Ontology Hub para OH-APP-10, OH-APP-22 y versions.js ENOENT; después continuar cierre A5.2 con AI Model Hub/Observer y evidencias finales.</t>
+          <t>Comunicar incidencias de Ontology Hub y reejecutar tras corrección del componente.</t>
         </is>
       </c>
     </row>
@@ -3332,12 +3332,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Automatizado alto / 27/27 passed en último Level 6 disponible; modelos reales FLARES/GTFS pendientes</t>
+          <t>Automatizado con baseline controlada / 32 de 32 casos trazados</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Level 6 ejecuta UI, functional, connector governance, model execution, benchmarking, mobility y Observer. Último resumen disponible: 27/27 passed.</t>
+          <t>Level 6 ejecuta UI, functional, connector governance, model execution, benchmarking, mobility y Observer. Último resumen disponible: 27/27 passed; queda generar evidencia final sin Kafka.</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -3347,12 +3347,12 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>FLARES/GTFS con modelos reales siguen dependiendo de la integración final de modelos externos; el model-server mantiene fixture determinista temporal.</t>
+          <t>FLARES/GTFS con modelos reales quedan como reemplazo futuro de la baseline controlada. El model-server mantiene contratos reproducibles para A5.2.</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>Mantener automatización actual y sustituir fixtures por modelos reales cuando estén disponibles.</t>
+          <t>Reejecutar Level 6 sin Kafka y sustituir endpoints controlados por modelos reales cuando estén disponibles.</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>PT5-MH-03, 08, 09, 10, 11, 16, 17, 18; DS-UI-AMH-01; MH-OBS-01/02.</t>
+          <t>PT5-MH-03, 08, 09, 10, 11, 16, 17, 18; DS-UI-AMH-01; MH-OBS-01..06.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -3436,12 +3436,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Implementado técnicamente / 22 de 23 casos trazados</t>
+          <t>Implementado técnicamente / 23 de 23 casos trazados</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Cobertura técnica real 22/23 (95.7%) con Automap fase 2 determinista y reutilización Ontology Hub incluidas; queda pendiente la revisión final de Level 6 sin Kafka y el registro de incidencias reales si aparecen.</t>
+          <t>Cobertura técnica real 23/23 (100.0%) confirmada por Level 6 2026-05-22; Automap fase 2, reutilización Ontology Hub, GTFS-Bench y UI mapping-editor pasaron.</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -3451,12 +3451,12 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>La integración explícita con Ontology Hub queda cubierta por mapping_validation y automap_execution. La revisión QA del conjunto del Virtualizador sigue pendiente de la ejecución final.</t>
+          <t>Sin pendientes técnicos vigentes del Virtualizador en la baseline A5.2. Mantener seguimiento solo si cambian los repos o despliegues del componente.</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Ejecutar Level 6 final y registrar únicamente incidencias reales del componente o del framework.</t>
+          <t>Conservar evidencia del experimento 2026-05-22 y reejecutar si se modifica el componente.</t>
         </is>
       </c>
     </row>
@@ -3757,12 +3757,12 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Pendiente inmediata tras revisión QA del Virtualizador</t>
+          <t>Ejecutado 2026-05-22 con fallos conocidos de Ontology Hub</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Dashboard unificado y JSON generados por ejecución sin fallos de framework; fallos de componente documentados.</t>
+          <t>Dashboard unificado generado; Newman, AI Model Hub y Semantic Virtualization pasaron. La spec 15 de AI Model Execution se corrigió y pasó en ejecución focalizada posterior. Persisten fallos conocidos de Ontology Hub.</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Requiere haber ejecutado niveles 3, 4 y 5 del adapter activo.</t>
+          <t>La ejecución completa queda en estado failed por incidencias de componente y por la spec 15 antes del fix. El fix de spec 15 fue validado de forma focalizada.</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Ejecutar Level 6 final sin Kafka y actualizar porcentajes si el Virtualizador queda validado.</t>
+          <t>Reejecutar Level 6 completo solo si se necesita dashboard final sin el fallo previo de spec 15; en cualquier caso Ontology Hub seguirá fallando hasta corregir OH-APP-10, OH-APP-22 y PT5-OH-13.</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Preparado como smoke UI/API; pendiente de integración final del componente</t>
+          <t>Automatizado con baseline controlada / pendiente evidencia final Level 6</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -4768,12 +4768,12 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>Observer UI/API aún no integrado en el entorno actual; los tests generan skips controlados.</t>
+          <t>Observer UI/API queda automatizado con eventos QA controlados; los skips solo aplican a entornos antiguos que no expongan la ruta Observer.</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>Tenemos la estrategia y smoke tests preparados; queda desbloquear rutas reales con equipo del componente/coordinación técnica.</t>
+          <t>Tenemos smoke UI, API journal, timeline, agreement evidence, benchmark evidence y participant summary preparados para evidencia final.</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Definido / parcialmente automatizado; pendiente dataset-endpoint real estable</t>
+          <t>Automatizado con baseline controlada; modelos reales FLARES quedan como evolución del componente</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
@@ -4892,12 +4892,12 @@
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Alinear con equipo del componente que dataset FLARES/modelo endpoint esten disponibles; los modelos concretos se decidiran segun el caso de uso y datos.</t>
+          <t>Level 6 publica FLARES bajo demanda, negocia el acceso y ejecuta payloads contra un endpoint model-server controlado; los modelos reales se sustituyen cuando estén disponibles.</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>Alineado con coordinación técnica: el foco no es XGBoost/Linear Regression/Decisión Tree, sino el caso lingüístico; el modelo queda como decisión técnica posterior.</t>
+          <t>El caso lingüístico queda defendible para A5.2 con baseline reproducible y trazabilidad a FLARES.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>Definido / automatización alta con fixtures; pendiente modelo real final si se exige inferencia live</t>
+          <t>Automatizado con baseline controlada; modelos reales GTFS quedan como evolución del componente</t>
         </is>
       </c>
       <c r="I18" s="9" t="inlineStr">
@@ -4955,12 +4955,12 @@
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>Confirmar con equipo del componente/coordinación técnica si el objetivo final sera estimación de llegada/delay u otro patron; ajustar modelo segun dataset.</t>
+          <t>Level 6 usa GTFS-Bench oficial, valida joins/benchmarking y ejecuta endpoints controlados de movilidad; el modelo real final se sustituye sin cambiar el contrato de prueba.</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>Alineado con coordinación técnica: el caso de movilidad guia dataset y validación; el modelo se elige después segun datos y metrica.</t>
+          <t>El caso de movilidad queda defendible para A5.2 con baseline reproducible y trazabilidad a GTFS-Bench.</t>
         </is>
       </c>
     </row>
@@ -7353,7 +7353,7 @@
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
+          <t>Level 6 2026-05-22: passed</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -7369,6 +7369,72 @@
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-05-22: OH-APP-15, OH-APP-16, OH-APP-17 y OH-APP-18 pasaron en la suite funcional completa; no mantener PT5-OH-05 como pendiente vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="27.9" customHeight="1" s="26">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-06</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Action logging</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Ontology Hub</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>non_functional</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>- The system exposes a functional auditing or logging mechanism</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Execute ontology operations.
+Paso 2: Query the audit trail.</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Actions are recorded for auditing</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>Baseline idempotente marcada 2026-05-07: failed</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Entregable E5.1 de validación
+Entregable técnico de Ontology Hub</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
 Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
@@ -7376,67 +7442,139 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="27.9" customHeight="1" s="26">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-06</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Action logging</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
+    <row r="13" ht="27.9" customHeight="1" s="26">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-07</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>RDF / OWL compatibility</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Ontology Hub</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>non_functional</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>interoperability</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>- The system exposes a functional auditing or logging mechanism</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Execute ontology operations.
-Paso 2: Query the audit trail.</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Actions are recorded for auditing</t>
-        </is>
-      </c>
-      <c r="I12" s="1" t="n"/>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
-        </is>
-      </c>
-      <c r="K12" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>- An RDF or OWL ontology is available to register</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Register an RDF or OWL ontology.
+Paso 2: Validate the semantic compatibility of the resource.</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>The ontology satisfies the semantic requirements</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="n"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Baseline idempotente marcada 2026-05-07: passed</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L12" s="9" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Ontology Hub</t>
         </is>
       </c>
-      <c r="M12" s="9" t="inlineStr">
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
+Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="27.9" customHeight="1" s="26">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-08</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Vocabulary search</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Ontology Hub</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>- Ontology Hub is deployed and reachable
+- The search API is available</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Execute a free-text search.
+Paso 2: Validate the response returned by the API or UI.</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Search results are coherent with the query</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>pt5_oh_08_term_search</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Baseline idempotente marcada 2026-05-07: passed</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Entregable E5.1 de validación
+Entregable técnico de Ontology Hub</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
 Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
@@ -7444,139 +7582,71 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27.9" customHeight="1" s="26">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-07</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>RDF / OWL compatibility</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
+    <row r="15" ht="27.9" customHeight="1" s="26">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-09</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Vocabulary filtering</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Ontology Hub</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>interoperability</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>- An RDF or OWL ontology is available to register</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Register an RDF or OWL ontology.
-Paso 2: Validate the semantic compatibility of the resource.</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>The ontology satisfies the semantic requirements</t>
-        </is>
-      </c>
-      <c r="I13" s="1" t="n"/>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>- Visible facets or filters exist in the catalog</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Filter by metadata and tags.
+Paso 2: Review the resulting set.</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Filtered results are correct</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/ontology_hub/integration/specs/pt5_oh_09_filters.spec.js</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Baseline idempotente marcada 2026-05-07: passed</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="K15" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L13" s="9" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Ontology Hub</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr">
-        <is>
-          <t>Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
-Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="27.9" customHeight="1" s="26">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-08</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Vocabulary search</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Ontology Hub</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>functional</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>- Ontology Hub is deployed and reachable
-- The search API is available</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Execute a free-text search.
-Paso 2: Validate the response returned by the API or UI.</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>Search results are coherent with the query</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>pt5_oh_08_term_search</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: passed</t>
-        </is>
-      </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework de validación
-Resultados estructurados JSON generados por la suite</t>
-        </is>
-      </c>
-      <c r="L14" s="9" t="inlineStr">
-        <is>
-          <t>Entregable E5.1 de validación
-Entregable técnico de Ontology Hub</t>
-        </is>
-      </c>
-      <c r="M14" s="9" t="inlineStr">
+      <c r="M15" s="9" t="inlineStr">
         <is>
           <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
 Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
@@ -7584,71 +7654,210 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="27.9" customHeight="1" s="26">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-09</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Vocabulary filtering</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+    <row r="16" ht="27.9" customHeight="1" s="26">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-10</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Version selection</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Ontology Hub</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>functional</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>- Visible facets or filters exist in the catalog</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Filter by metadata and tags.
-Paso 2: Review the resulting set.</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>Filtered results are correct</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>validation/components/ontology_hub/integration/specs/pt5_oh_09_filters.spec.js</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: passed</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>- At least one ontology exists with multiple versions</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Open an ontology with multiple versions.
+Paso 2: Select a specific version.</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>The requested version is displayed</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/ontology_hub/integration/specs/pt5_oh_10_versions.spec.js</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>Level 6 2026-05-22: passed</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Ontology Hub</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-05-22: OH-APP-11, OH-APP-12 y OH-APP-13 pasaron; el bloque de versiones no queda como pendiente vigente en esta ejecución.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="27.9" customHeight="1" s="26">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-11</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Complete ontology visualization</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Ontology Hub</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>- An ontology detail page is accessible</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Open the detail page of an ontology.
+Paso 2: Review metadata, code, and graphical elements.</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Metadata, code, and graphics are visible</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/ontology_hub/integration/specs/pt5_oh_11_vocab_detail.spec.js</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>Level 6 2026-05-22: passed</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>Entregable E5.1 de validación
+Entregable técnico de Ontology Hub</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-05-22: OH-APP-05 pasó; la ficha de ontología y descarga .n3 quedan validadas en la ejecución final sin Kafka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="27.9" customHeight="1" s="26">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-12</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Ontology statistics</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Ontology Hub</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>- The detail page or catalog shows statistics or popularity</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Check statistics and popularity for an ontology.</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Metrics are visible as defined</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>validation/components/ontology_hub/integration/specs/pt5_oh_12_statistics.spec.js</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Baseline idempotente marcada 2026-05-07: passed</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Evidencia generada por el framework de validación
+Resultados estructurados JSON generados por la suite</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Entregable E5.1 de validación
+Entregable técnico de Ontology Hub</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
 Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
@@ -7656,290 +7865,73 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27.9" customHeight="1" s="26">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-10</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Version selection</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
+    <row r="19" ht="27.9" customHeight="1" s="26">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>PT5-OH-13</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>SPARQL query</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Ontology Hub</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>functional</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>interoperability</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>- At least one ontology exists with multiple versions</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Open an ontology with multiple versions.
-Paso 2: Select a specific version.</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>The requested version is displayed</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>validation/components/ontology_hub/integration/specs/pt5_oh_10_versions.spec.js</t>
-        </is>
-      </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
-        </is>
-      </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>- The instance exposes SPARQL access or a query page</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Paso 1: Execute a SPARQL query.
+Paso 2: Validate the obtained response.</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>The query returns valid results</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>pt5_oh_13_sparql_access</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Level 6 2026-05-22: failed por issue de componente</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>Evidencia generada por el framework de validación
 Resultados estructurados JSON generados por la suite</t>
         </is>
       </c>
-      <c r="L16" s="9" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>Entregable E5.1 de validación
 Entregable técnico de Ontology Hub</t>
         </is>
       </c>
-      <c r="M16" s="9" t="inlineStr">
-        <is>
-          <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
-Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
-Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="27.9" customHeight="1" s="26">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-11</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Complete ontology visualization</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Ontology Hub</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>functional</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>- An ontology detail page is accessible</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Open the detail page of an ontology.
-Paso 2: Review metadata, code, and graphical elements.</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Metadata, code, and graphics are visible</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>validation/components/ontology_hub/integration/specs/pt5_oh_11_vocab_detail.spec.js</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: failed</t>
-        </is>
-      </c>
-      <c r="K17" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework de validación
-Resultados estructurados JSON generados por la suite</t>
-        </is>
-      </c>
-      <c r="L17" s="9" t="inlineStr">
-        <is>
-          <t>Entregable E5.1 de validación
-Entregable técnico de Ontology Hub</t>
-        </is>
-      </c>
-      <c r="M17" s="9" t="inlineStr">
-        <is>
-          <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
-Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
-Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="27.9" customHeight="1" s="26">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-12</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Ontology statistics</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Ontology Hub</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>functional</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>- The detail page or catalog shows statistics or popularity</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Check statistics and popularity for an ontology.</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Metrics are visible as defined</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>validation/components/ontology_hub/integration/specs/pt5_oh_12_statistics.spec.js</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: passed</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework de validación
-Resultados estructurados JSON generados por la suite</t>
-        </is>
-      </c>
-      <c r="L18" s="9" t="inlineStr">
-        <is>
-          <t>Entregable E5.1 de validación
-Entregable técnico de Ontology Hub</t>
-        </is>
-      </c>
-      <c r="M18" s="9" t="inlineStr">
-        <is>
-          <t>Baseline afectada por crash real de Ontology Hub en flujo de versiones; revisar issue de componente ENOENT versions.js y distinguir fallos directos de cascada.
-Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
-Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="27.9" customHeight="1" s="26">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>PT5-OH-13</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>SPARQL query</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Ontology Hub</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>interoperability</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>- The instance exposes SPARQL access or a query page</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Paso 1: Execute a SPARQL query.
-Paso 2: Validate the obtained response.</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>The query returns valid results</t>
-        </is>
-      </c>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>pt5_oh_13_sparql_access</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>Baseline idempotente marcada 2026-05-07: skipped</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="inlineStr">
-        <is>
-          <t>Evidencia generada por el framework de validación
-Resultados estructurados JSON generados por la suite</t>
-        </is>
-      </c>
-      <c r="L19" s="9" t="inlineStr">
-        <is>
-          <t>Entregable E5.1 de validación
-Entregable técnico de Ontology Hub</t>
-        </is>
-      </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>A real SPARQL query is executed against the public SPARQL endpoint using the class URI exposed by the current seeded search result.
-Estado actualizado desde la baseline funcional marcada 2026-05-07 con trazabilidad OH-APP -&gt; PT5-OH.
-Estado actualizado desde la baseline funcional idempotente marcada 2026-05-07.</t>
+          <t>La integración API ejecutó pt5_oh_13_sparql_access y recibió HTTP 502 en el endpoint SPARQL público. Clasificar como incidencia del componente/servicio Ontology Hub, no como fallo de framework.</t>
         </is>
       </c>
     </row>
@@ -9080,12 +9072,7 @@
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Issue conocido observado en la ejecución real: requiere validación por desarrolladores del componente antes de cierre total. Mapeo PT5 en nueva evidencia: PT5-OH-02.
-Fallo directo antes del crash de versiones; mantener como issue de componente.
-Fallo en cascada en esta baseline porque OH-APP-04 no genero el estado compartido oh-app-04-repository-vocabulary; no hubo restart nuevo del pod.
-Fallo vigente: los metadatos/tags editados no quedan visibles a tiempo en la ficha tras guardar.
-Se aumento la espera/refresco a 60s; la ficha sigue sin mostrar Vocabularies ni ADMIN TEST, por lo que no parece un timeout corto del framework.
-Última baseline 2026-05-07 19:27:24: failed. Tras Save, la ficha sigue mostrando Services/Admin y no Vocabularies/ADMIN TEST; se clasifica como issue de componente.</t>
+          <t>Actualizado 2026-05-22: sigue fallando. Tras guardar, Ontology Hub no expone Vocabularies ni ADMIN TEST metadata update después de 180s; se clasifica como issue de persistencia/reindexado del componente.</t>
         </is>
       </c>
     </row>
@@ -9641,11 +9628,7 @@
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>Issue conocido observado en la ejecución real: requiere validación por desarrolladores del componente antes de cierre total. Mapeo PT5 en nueva evidencia: PT5-OH-05.
-Fallo en cascada tras crash de Ontology Hub/port-forward perdido; no tratar como fallo independiente del framework.
-Fallo funcional independiente: la pagina de administracion de usuarios devolvio 500 y bloquea la promocion a admin.
-Fallo vigente: pagina de administracion de usuarios devuelve 500 y bloquea promocion a admin.
-Última baseline 2026-05-07 19:27:24: passed dentro de la suite completa 25/27.</t>
+          <t>Actualizado 2026-05-22: OH-APP-17 pasó en Level 6; la promoción de usuario a admin y visibilidad de + USER no queda como pendiente vigente. Mantener solo como antecedente histórico de ejecuciones anteriores.</t>
         </is>
       </c>
     </row>
@@ -10040,11 +10023,7 @@
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Issue conocido observado en la ejecución real: requiere validación por desarrolladores del componente antes de cierre total. Mapeo PT5 en nueva evidencia: PT5-OH-06, PT5-OH-14.
-Fallo en cascada tras crash de Ontology Hub/port-forward perdido; no tratar como fallo independiente del framework.
-Fallo funcional independiente: la pagina Patterns devolvio 500 y no se pudo generar el zip.
-Fallo vigente: pagina Patterns devuelve 500 y no genera ZIP.
-Última baseline 2026-05-07 19:27:24: failed. /dataset/patterns devuelve 500 antes de interactuar con Select All o generar el ZIP; se clasifica como issue de componente.</t>
+          <t>Actualizado 2026-05-22: sigue fallando. /dataset/patterns devuelve 500 y bloquea la generación del ZIP; FOOPS y Themis sí pasaron, por lo que el fallo queda localizado en Patterns.</t>
         </is>
       </c>
     </row>
@@ -10768,7 +10747,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
@@ -10839,7 +10818,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -10981,7 +10960,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -11052,7 +11031,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -11123,7 +11102,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -11193,7 +11172,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
@@ -11786,7 +11765,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Automatizado parcial UI / Level 6 por defecto</t>
+          <t>Automatizado UI/API / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
@@ -12076,7 +12055,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Parcial automatizado / Level 6 por defecto</t>
+          <t>Automatizado baseline controlado / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
@@ -12093,7 +12072,7 @@
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>Slice lingüístico actual mantiene evidencia reproducible; ampliar con nuevos flujos si el componente expone más funcionalidades.</t>
+          <t>Baseline lingüística reproducible: publica FLARES bajo demanda, negocia acceso, prepara benchmark y ejecuta payload FLARES mediante model-server controlado. Los modelos reales FLARES son reemplazables y no bloquean la baseline A5.2.</t>
         </is>
       </c>
     </row>
@@ -12461,7 +12440,7 @@
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>Automatizado parcial / mapped / Level 6 dataspace</t>
+          <t>Automatizado / mapped / Level 6 dataspace</t>
         </is>
       </c>
       <c r="K30" s="9" t="inlineStr">
@@ -12480,7 +12459,7 @@
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>El Browser registra evidencia observable cuando el backend Observer está disponible; si no, deja subcheck controlado sin bloquear el resto de Level 6.</t>
+          <t>Browser registra evidencia observable cuando el backend Observer está disponible; si no, deja subcheck controlado sin bloquear descubrimiento.</t>
         </is>
       </c>
     </row>
@@ -12539,7 +12518,7 @@
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>Automatizado parcial / mapped / Level 6 por defecto</t>
+          <t>Automatizado / mapped / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
@@ -12558,7 +12537,7 @@
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>La ejecución local y externa genera correlationId/evidencia cuando Observer está disponible; la inferencia real queda cubierta por runner API HttpData.</t>
+          <t>Ejecución local y externa generan correlationId/evidencia cuando Observer está disponible; la inferencia A5.2 queda cubierta por HttpData y model-server controlado.</t>
         </is>
       </c>
     </row>
@@ -12615,7 +12594,7 @@
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>Automatizado parcial / mapped / Level 6 por defecto</t>
+          <t>Automatizado / mapped / Level 6 por defecto</t>
         </is>
       </c>
       <c r="K32" s="9" t="inlineStr">
@@ -12634,7 +12613,7 @@
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>El benchmarking registra benchmarkRunId/evidencia cuando el Observer está disponible; conserva subcheck controlado si el backend no expone la ruta.</t>
+          <t>Benchmarking registra benchmarkRunId/evidencia cuando Observer está disponible; conserva subcheck controlado si el backend no expone la ruta.</t>
         </is>
       </c>
     </row>
@@ -12710,7 +12689,7 @@
       </c>
       <c r="M33" s="9" t="inlineStr">
         <is>
-          <t>El resumen de participante queda cubierto por UI y API con eventos QA controlados, hashes y contadores sin payloads sensibles.</t>
+          <t>Resumen de participante cubierto por UI y API con eventos QA controlados, hashes y contadores sin payloads sensibles.</t>
         </is>
       </c>
     </row>
@@ -15076,7 +15055,7 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>El workbook refleja 22/23 (95.7%) como avance técnico vigente del Virtualizador.</t>
+          <t>El workbook refleja 23/23 (100.0%) como avance técnico vigente del Virtualizador.</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr">
@@ -15087,7 +15066,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Estado real registrado con Automap fase 2 determinista y reutilización Ontology Hub</t>
+          <t>Estado real registrado con Level 6 2026-05-22: UI mapping-editor, API, GTFS-Bench, Automap y reutilización Ontology Hub pasaron.</t>
         </is>
       </c>
       <c r="K34" s="9" t="inlineStr">
@@ -15104,7 +15083,7 @@
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>Pendientes principales: integración específica con Ontology Hub y revisión final de ejecución Level 6 sin Kafka.</t>
+          <t>Level 6 2026-05-22 confirma 29/29 en component validation y 11/11 en UI del Virtualizador; no quedan pendientes técnicos vigentes del componente en la baseline A5.2.</t>
         </is>
       </c>
     </row>
@@ -15923,12 +15902,12 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Actualizado 2026-05-18: MH-OBS-01 y MH-OBS-02 quedan automated/mapped; MH-OBS-03..06 siguen planned como ampliaciones futuras.</t>
+          <t>Actualizado 2026-05-22: MH-OBS-01..06 quedan automated/mapped. Observer cubre home, journal API, Browser evidence, Execution evidence, Benchmark evidence y Participant summary con subchecks controlados cuando un entorno antiguo no expone la ruta.</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Usar para explicar que Observer/Clearing House ya está integrado en la arquitectura de pruebas y que la evidencia final depende de reejecutar nivel 6.</t>
+          <t>Usar para explicar que Observer/Clearing House ya está integrado en la arquitectura de pruebas; la evidencia final depende de reejecutar nivel 6 sin Kafka.</t>
         </is>
       </c>
     </row>

</xml_diff>